<commit_message>
Business plan v6: update funding to £14k equity and Bedfordshire pilot status
Founders £3,000, friends & family £3,000, Nigerian company £8,000 (equity).
Model, cash flow, balance sheet, use of funds and narrative updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146q3FtAYmgQ1rtNsNNpdiD
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -573,32 +573,52 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Founder share capital (£)</t>
+          <t>Founders' opening capital (£)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Licence billing</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Annual in advance, 30-day terms, revenue recognised monthly</t>
-        </is>
+          <t>Friends &amp; family equity (£, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Nigerian company equity (£, Nov 2026)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Licence billing</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Annual in advance, 30-day terms, revenue recognised monthly</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Not registered — taxable turnover below £90,000 in base case</t>
         </is>
@@ -615,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN54"/>
+  <dimension ref="A1:AN55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3010,7 +3030,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>0</v>
@@ -3106,7 +3126,7 @@
         <v>0</v>
       </c>
       <c r="AL22" s="4" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="AM22" s="4" t="n">
         <v>600</v>
@@ -3258,7 +3278,7 @@
         <v>71.55</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>373.23</v>
+        <v>573.23</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>74.08</v>
@@ -3354,7 +3374,7 @@
         <v>463.22</v>
       </c>
       <c r="AL24" s="4" t="n">
-        <v>1189.57</v>
+        <v>1389.57</v>
       </c>
       <c r="AM24" s="4" t="n">
         <v>2670.96</v>
@@ -3382,7 +3402,7 @@
         <v>-56.58</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>-353.27</v>
+        <v>-553.27</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>-54.12</v>
@@ -3478,7 +3498,7 @@
         <v>4714.41</v>
       </c>
       <c r="AL25" s="4" t="n">
-        <v>-620.08</v>
+        <v>-820.08</v>
       </c>
       <c r="AM25" s="4" t="n">
         <v>19439.96</v>
@@ -4160,40 +4180,40 @@
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>128</v>
+        <v>240</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>112</v>
+        <v>210</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>96</v>
+        <v>180</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>104</v>
+        <v>195</v>
       </c>
       <c r="N32" s="4" t="n">
         <v>560</v>
@@ -4268,7 +4288,7 @@
         <v>780</v>
       </c>
       <c r="AL32" s="4" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="AM32" s="4" t="n">
         <v>3500</v>
@@ -5276,40 +5296,40 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>-481.27</v>
+        <v>-593.27</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>-585.71</v>
+        <v>-683.71</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>-271.23</v>
+        <v>-341.23</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>-607.58</v>
+        <v>-635.58</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>-584.27</v>
+        <v>-868.27</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-261.12</v>
+        <v>-324.12</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-241.27</v>
+        <v>-290.27</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>-201.64</v>
+        <v>-236.64</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>-193.95</v>
+        <v>-221.95</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>-186.15</v>
+        <v>-207.15</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>-137.32</v>
+        <v>-158.32</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>-268.57</v>
+        <v>-359.57</v>
       </c>
       <c r="N41" s="4" t="n">
         <v>-1341</v>
@@ -5384,7 +5404,7 @@
         <v>897.25</v>
       </c>
       <c r="AL41" s="4" t="n">
-        <v>-4020.08</v>
+        <v>-4920.08</v>
       </c>
       <c r="AM41" s="4" t="n">
         <v>9678.940000000001</v>
@@ -5409,40 +5429,40 @@
         <v>0</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="J42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="O42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="P42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="Q42" s="4" t="n">
         <v>41.67</v>
@@ -5508,10 +5528,10 @@
         <v>75</v>
       </c>
       <c r="AL42" s="4" t="n">
-        <v>0</v>
+        <v>150.03</v>
       </c>
       <c r="AM42" s="4" t="n">
-        <v>375.03</v>
+        <v>425.04</v>
       </c>
       <c r="AN42" s="4" t="n">
         <v>866.67</v>
@@ -5524,49 +5544,49 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>-481.27</v>
+        <v>-593.27</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>-585.71</v>
+        <v>-683.71</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>-271.23</v>
+        <v>-341.23</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>-607.58</v>
+        <v>-652.24</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>-584.27</v>
+        <v>-884.9400000000001</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>-261.12</v>
+        <v>-340.79</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>-241.27</v>
+        <v>-306.93</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>-201.64</v>
+        <v>-253.31</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>-193.95</v>
+        <v>-238.62</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>-186.15</v>
+        <v>-223.82</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>-137.32</v>
+        <v>-174.98</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>-268.57</v>
+        <v>-376.24</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>-1341</v>
+        <v>-1357.66</v>
       </c>
       <c r="O43" s="4" t="n">
-        <v>273.05</v>
+        <v>256.39</v>
       </c>
       <c r="P43" s="4" t="n">
-        <v>1066.2</v>
+        <v>1049.53</v>
       </c>
       <c r="Q43" s="4" t="n">
         <v>248.87</v>
@@ -5632,10 +5652,10 @@
         <v>822.25</v>
       </c>
       <c r="AL43" s="4" t="n">
-        <v>-4020.08</v>
+        <v>-5070.08</v>
       </c>
       <c r="AM43" s="4" t="n">
-        <v>9303.93</v>
+        <v>9253.940000000001</v>
       </c>
       <c r="AN43" s="4" t="n">
         <v>3865.48</v>
@@ -5951,7 +5971,7 @@
         <v>0</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F47" s="4" t="n">
         <v>0</v>
@@ -5987,7 +6007,7 @@
         <v>0</v>
       </c>
       <c r="Q47" s="4" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="R47" s="4" t="n">
         <v>0</v>
@@ -6050,10 +6070,10 @@
         <v>0</v>
       </c>
       <c r="AL47" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="AM47" s="4" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="AN47" s="4" t="n">
         <v>1200</v>
@@ -6165,7 +6185,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>790</v>
+        <v>619</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -6180,555 +6200,555 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>790</v>
+        <v>619</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Total payments</t>
+          <t>Equity investment received</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
-        <v>481.27</v>
+        <v>0</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>585.71</v>
+        <v>3000</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>286.2</v>
+        <v>8000</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>622.55</v>
+        <v>0</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>604.23</v>
+        <v>0</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>281.08</v>
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>266.22</v>
+        <v>0</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>276.58</v>
+        <v>0</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>268.89</v>
+        <v>0</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>261.09</v>
+        <v>0</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>262.25</v>
+        <v>0</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>393.5</v>
+        <v>0</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>1530.89</v>
+        <v>0</v>
       </c>
       <c r="O49" s="4" t="n">
-        <v>1598.47</v>
+        <v>0</v>
       </c>
       <c r="P49" s="4" t="n">
-        <v>865.3</v>
+        <v>0</v>
       </c>
       <c r="Q49" s="4" t="n">
-        <v>3140.96</v>
+        <v>0</v>
       </c>
       <c r="R49" s="4" t="n">
-        <v>943.8</v>
+        <v>0</v>
       </c>
       <c r="S49" s="4" t="n">
-        <v>844.95</v>
+        <v>0</v>
       </c>
       <c r="T49" s="4" t="n">
-        <v>778.54</v>
+        <v>0</v>
       </c>
       <c r="U49" s="4" t="n">
-        <v>710.5599999999999</v>
+        <v>0</v>
       </c>
       <c r="V49" s="4" t="n">
-        <v>677.99</v>
+        <v>0</v>
       </c>
       <c r="W49" s="4" t="n">
-        <v>643.95</v>
+        <v>0</v>
       </c>
       <c r="X49" s="4" t="n">
-        <v>644.42</v>
+        <v>0</v>
       </c>
       <c r="Y49" s="4" t="n">
-        <v>1552.14</v>
+        <v>0</v>
       </c>
       <c r="Z49" s="4" t="n">
-        <v>5173.8</v>
+        <v>0</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>5335.38</v>
+        <v>0</v>
       </c>
       <c r="AB49" s="4" t="n">
-        <v>3911.52</v>
+        <v>0</v>
       </c>
       <c r="AC49" s="4" t="n">
-        <v>4689.67</v>
+        <v>0</v>
       </c>
       <c r="AD49" s="4" t="n">
-        <v>4054.94</v>
+        <v>0</v>
       </c>
       <c r="AE49" s="4" t="n">
-        <v>4286.42</v>
+        <v>0</v>
       </c>
       <c r="AF49" s="4" t="n">
-        <v>4436.39</v>
+        <v>0</v>
       </c>
       <c r="AG49" s="4" t="n">
-        <v>3722.04</v>
+        <v>0</v>
       </c>
       <c r="AH49" s="4" t="n">
-        <v>3666.24</v>
+        <v>0</v>
       </c>
       <c r="AI49" s="4" t="n">
-        <v>4398.1</v>
+        <v>0</v>
       </c>
       <c r="AJ49" s="4" t="n">
-        <v>3610.96</v>
+        <v>0</v>
       </c>
       <c r="AK49" s="4" t="n">
-        <v>4280.39</v>
+        <v>0</v>
       </c>
       <c r="AL49" s="4" t="n">
-        <v>4589.57</v>
+        <v>11000</v>
       </c>
       <c r="AM49" s="4" t="n">
-        <v>13931.97</v>
+        <v>0</v>
       </c>
       <c r="AN49" s="4" t="n">
-        <v>51565.85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Net cash flow</t>
+          <t>Total payments</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>-481.27</v>
+        <v>593.27</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>-585.71</v>
+        <v>683.71</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>-271.23</v>
+        <v>356.2</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>-607.58</v>
+        <v>1250.55</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>-584.27</v>
+        <v>888.23</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>-261.12</v>
+        <v>344.08</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>-241.27</v>
+        <v>315.22</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>-201.64</v>
+        <v>311.58</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>-193.95</v>
+        <v>296.89</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>-186.15</v>
+        <v>282.09</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>-137.32</v>
+        <v>283.25</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>-268.57</v>
+        <v>484.5</v>
       </c>
       <c r="N50" s="4" t="n">
-        <v>-1341</v>
+        <v>1530.89</v>
       </c>
       <c r="O50" s="4" t="n">
-        <v>18606.39</v>
+        <v>1598.47</v>
       </c>
       <c r="P50" s="4" t="n">
-        <v>-600.47</v>
+        <v>865.3</v>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>-2876.13</v>
+        <v>2540.96</v>
       </c>
       <c r="R50" s="4" t="n">
-        <v>-668.99</v>
+        <v>943.8</v>
       </c>
       <c r="S50" s="4" t="n">
-        <v>-510.17</v>
+        <v>844.95</v>
       </c>
       <c r="T50" s="4" t="n">
-        <v>-438.77</v>
+        <v>778.54</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>-370.79</v>
+        <v>710.5599999999999</v>
       </c>
       <c r="V50" s="4" t="n">
-        <v>-288.23</v>
+        <v>677.99</v>
       </c>
       <c r="W50" s="4" t="n">
-        <v>-254.19</v>
+        <v>643.95</v>
       </c>
       <c r="X50" s="4" t="n">
-        <v>-259.65</v>
+        <v>644.42</v>
       </c>
       <c r="Y50" s="4" t="n">
-        <v>-1152.4</v>
+        <v>1552.14</v>
       </c>
       <c r="Z50" s="4" t="n">
-        <v>15330.82</v>
+        <v>5173.8</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>15209.16</v>
+        <v>5335.38</v>
       </c>
       <c r="AB50" s="4" t="n">
-        <v>-3292.04</v>
+        <v>3911.52</v>
       </c>
       <c r="AC50" s="4" t="n">
-        <v>-4070.19</v>
+        <v>4689.67</v>
       </c>
       <c r="AD50" s="4" t="n">
-        <v>-3355.53</v>
+        <v>4054.94</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>-3622.03</v>
+        <v>4286.42</v>
       </c>
       <c r="AF50" s="4" t="n">
-        <v>8287.969999999999</v>
+        <v>4436.39</v>
       </c>
       <c r="AG50" s="4" t="n">
-        <v>-2992.69</v>
+        <v>3722.04</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>-2891.89</v>
+        <v>3666.24</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>-3628.74</v>
+        <v>4227.1</v>
       </c>
       <c r="AJ50" s="4" t="n">
-        <v>-2796.6</v>
+        <v>3610.96</v>
       </c>
       <c r="AK50" s="4" t="n">
-        <v>-3436.09</v>
+        <v>4280.39</v>
       </c>
       <c r="AL50" s="4" t="n">
-        <v>-4020.08</v>
+        <v>6089.57</v>
       </c>
       <c r="AM50" s="4" t="n">
-        <v>9845.6</v>
+        <v>13331.97</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>8742.15</v>
+        <v>51394.85</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Net cash flow</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n">
+        <v>-593.27</v>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>2316.29</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>7658.77</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>-1235.58</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>-868.27</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>-324.12</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>-290.27</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>-236.64</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>-221.95</v>
+      </c>
+      <c r="K51" s="4" t="n">
+        <v>-207.15</v>
+      </c>
+      <c r="L51" s="4" t="n">
+        <v>-158.32</v>
+      </c>
+      <c r="M51" s="4" t="n">
+        <v>-359.57</v>
+      </c>
+      <c r="N51" s="4" t="n">
+        <v>-1341</v>
+      </c>
+      <c r="O51" s="4" t="n">
+        <v>18606.39</v>
+      </c>
+      <c r="P51" s="4" t="n">
+        <v>-600.47</v>
+      </c>
+      <c r="Q51" s="4" t="n">
+        <v>-2276.13</v>
+      </c>
+      <c r="R51" s="4" t="n">
+        <v>-668.99</v>
+      </c>
+      <c r="S51" s="4" t="n">
+        <v>-510.17</v>
+      </c>
+      <c r="T51" s="4" t="n">
+        <v>-438.77</v>
+      </c>
+      <c r="U51" s="4" t="n">
+        <v>-370.79</v>
+      </c>
+      <c r="V51" s="4" t="n">
+        <v>-288.23</v>
+      </c>
+      <c r="W51" s="4" t="n">
+        <v>-254.19</v>
+      </c>
+      <c r="X51" s="4" t="n">
+        <v>-259.65</v>
+      </c>
+      <c r="Y51" s="4" t="n">
+        <v>-1152.4</v>
+      </c>
+      <c r="Z51" s="4" t="n">
+        <v>15330.82</v>
+      </c>
+      <c r="AA51" s="4" t="n">
+        <v>15209.16</v>
+      </c>
+      <c r="AB51" s="4" t="n">
+        <v>-3292.04</v>
+      </c>
+      <c r="AC51" s="4" t="n">
+        <v>-4070.19</v>
+      </c>
+      <c r="AD51" s="4" t="n">
+        <v>-3355.53</v>
+      </c>
+      <c r="AE51" s="4" t="n">
+        <v>-3622.03</v>
+      </c>
+      <c r="AF51" s="4" t="n">
+        <v>8287.969999999999</v>
+      </c>
+      <c r="AG51" s="4" t="n">
+        <v>-2992.69</v>
+      </c>
+      <c r="AH51" s="4" t="n">
+        <v>-2891.89</v>
+      </c>
+      <c r="AI51" s="4" t="n">
+        <v>-3457.74</v>
+      </c>
+      <c r="AJ51" s="4" t="n">
+        <v>-2796.6</v>
+      </c>
+      <c r="AK51" s="4" t="n">
+        <v>-3436.09</v>
+      </c>
+      <c r="AL51" s="4" t="n">
+        <v>5479.92</v>
+      </c>
+      <c r="AM51" s="4" t="n">
+        <v>10445.6</v>
+      </c>
+      <c r="AN51" s="4" t="n">
+        <v>8913.15</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Closing cash</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n">
-        <v>5518.73</v>
-      </c>
-      <c r="C51" s="4" t="n">
-        <v>4933.02</v>
-      </c>
-      <c r="D51" s="4" t="n">
-        <v>4661.79</v>
-      </c>
-      <c r="E51" s="4" t="n">
-        <v>4054.21</v>
-      </c>
-      <c r="F51" s="4" t="n">
-        <v>3469.94</v>
-      </c>
-      <c r="G51" s="4" t="n">
-        <v>3208.82</v>
-      </c>
-      <c r="H51" s="4" t="n">
-        <v>2967.55</v>
-      </c>
-      <c r="I51" s="4" t="n">
-        <v>2765.91</v>
-      </c>
-      <c r="J51" s="4" t="n">
-        <v>2571.96</v>
-      </c>
-      <c r="K51" s="4" t="n">
-        <v>2385.81</v>
-      </c>
-      <c r="L51" s="4" t="n">
-        <v>2248.49</v>
-      </c>
-      <c r="M51" s="4" t="n">
-        <v>1979.92</v>
-      </c>
-      <c r="N51" s="4" t="n">
-        <v>638.92</v>
-      </c>
-      <c r="O51" s="4" t="n">
-        <v>19245.31</v>
-      </c>
-      <c r="P51" s="4" t="n">
-        <v>18644.84</v>
-      </c>
-      <c r="Q51" s="4" t="n">
-        <v>15768.72</v>
-      </c>
-      <c r="R51" s="4" t="n">
-        <v>15099.72</v>
-      </c>
-      <c r="S51" s="4" t="n">
-        <v>14589.56</v>
-      </c>
-      <c r="T51" s="4" t="n">
-        <v>14150.79</v>
-      </c>
-      <c r="U51" s="4" t="n">
-        <v>13780</v>
-      </c>
-      <c r="V51" s="4" t="n">
-        <v>13491.77</v>
-      </c>
-      <c r="W51" s="4" t="n">
-        <v>13237.58</v>
-      </c>
-      <c r="X51" s="4" t="n">
-        <v>12977.94</v>
-      </c>
-      <c r="Y51" s="4" t="n">
-        <v>11825.53</v>
-      </c>
-      <c r="Z51" s="4" t="n">
-        <v>27156.35</v>
-      </c>
-      <c r="AA51" s="4" t="n">
-        <v>42365.51</v>
-      </c>
-      <c r="AB51" s="4" t="n">
-        <v>39073.47</v>
-      </c>
-      <c r="AC51" s="4" t="n">
-        <v>35003.28</v>
-      </c>
-      <c r="AD51" s="4" t="n">
-        <v>31647.75</v>
-      </c>
-      <c r="AE51" s="4" t="n">
-        <v>28025.72</v>
-      </c>
-      <c r="AF51" s="4" t="n">
-        <v>36313.69</v>
-      </c>
-      <c r="AG51" s="4" t="n">
-        <v>33321</v>
-      </c>
-      <c r="AH51" s="4" t="n">
-        <v>30429.1</v>
-      </c>
-      <c r="AI51" s="4" t="n">
-        <v>26800.36</v>
-      </c>
-      <c r="AJ51" s="4" t="n">
-        <v>24003.76</v>
-      </c>
-      <c r="AK51" s="4" t="n">
-        <v>20567.68</v>
-      </c>
-      <c r="AL51" s="4" t="n">
-        <v>1979.92</v>
-      </c>
-      <c r="AM51" s="4" t="n">
-        <v>11825.53</v>
-      </c>
-      <c r="AN51" s="4" t="n">
-        <v>20567.68</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="B52" s="4" t="n">
+        <v>2406.73</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>4723.02</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>12381.79</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>11146.21</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>10277.94</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>9953.82</v>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>9663.549999999999</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>9426.91</v>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>9204.959999999999</v>
+      </c>
+      <c r="K52" s="4" t="n">
+        <v>8997.809999999999</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>8839.49</v>
+      </c>
+      <c r="M52" s="4" t="n">
+        <v>8479.92</v>
+      </c>
+      <c r="N52" s="4" t="n">
+        <v>7138.92</v>
+      </c>
+      <c r="O52" s="4" t="n">
+        <v>25745.31</v>
+      </c>
+      <c r="P52" s="4" t="n">
+        <v>25144.84</v>
+      </c>
+      <c r="Q52" s="4" t="n">
+        <v>22868.72</v>
+      </c>
+      <c r="R52" s="4" t="n">
+        <v>22199.72</v>
+      </c>
+      <c r="S52" s="4" t="n">
+        <v>21689.56</v>
+      </c>
+      <c r="T52" s="4" t="n">
+        <v>21250.79</v>
+      </c>
+      <c r="U52" s="4" t="n">
+        <v>20880</v>
+      </c>
+      <c r="V52" s="4" t="n">
+        <v>20591.77</v>
+      </c>
+      <c r="W52" s="4" t="n">
+        <v>20337.58</v>
+      </c>
+      <c r="X52" s="4" t="n">
+        <v>20077.94</v>
+      </c>
+      <c r="Y52" s="4" t="n">
+        <v>18925.53</v>
+      </c>
+      <c r="Z52" s="4" t="n">
+        <v>34256.35</v>
+      </c>
+      <c r="AA52" s="4" t="n">
+        <v>49465.51</v>
+      </c>
+      <c r="AB52" s="4" t="n">
+        <v>46173.47</v>
+      </c>
+      <c r="AC52" s="4" t="n">
+        <v>42103.28</v>
+      </c>
+      <c r="AD52" s="4" t="n">
+        <v>38747.75</v>
+      </c>
+      <c r="AE52" s="4" t="n">
+        <v>35125.72</v>
+      </c>
+      <c r="AF52" s="4" t="n">
+        <v>43413.69</v>
+      </c>
+      <c r="AG52" s="4" t="n">
+        <v>40421</v>
+      </c>
+      <c r="AH52" s="4" t="n">
+        <v>37529.1</v>
+      </c>
+      <c r="AI52" s="4" t="n">
+        <v>34071.36</v>
+      </c>
+      <c r="AJ52" s="4" t="n">
+        <v>31274.76</v>
+      </c>
+      <c r="AK52" s="4" t="n">
+        <v>27838.68</v>
+      </c>
+      <c r="AL52" s="4" t="n">
+        <v>8479.92</v>
+      </c>
+      <c r="AM52" s="4" t="n">
+        <v>18925.53</v>
+      </c>
+      <c r="AN52" s="4" t="n">
+        <v>27838.68</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>TEAM</t>
         </is>
       </c>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
-      <c r="K52" s="4" t="n"/>
-      <c r="L52" s="4" t="n"/>
-      <c r="M52" s="4" t="n"/>
-      <c r="N52" s="4" t="n"/>
-      <c r="O52" s="4" t="n"/>
-      <c r="P52" s="4" t="n"/>
-      <c r="Q52" s="4" t="n"/>
-      <c r="R52" s="4" t="n"/>
-      <c r="S52" s="4" t="n"/>
-      <c r="T52" s="4" t="n"/>
-      <c r="U52" s="4" t="n"/>
-      <c r="V52" s="4" t="n"/>
-      <c r="W52" s="4" t="n"/>
-      <c r="X52" s="4" t="n"/>
-      <c r="Y52" s="4" t="n"/>
-      <c r="Z52" s="4" t="n"/>
-      <c r="AA52" s="4" t="n"/>
-      <c r="AB52" s="4" t="n"/>
-      <c r="AC52" s="4" t="n"/>
-      <c r="AD52" s="4" t="n"/>
-      <c r="AE52" s="4" t="n"/>
-      <c r="AF52" s="4" t="n"/>
-      <c r="AG52" s="4" t="n"/>
-      <c r="AH52" s="4" t="n"/>
-      <c r="AI52" s="4" t="n"/>
-      <c r="AJ52" s="4" t="n"/>
-      <c r="AK52" s="4" t="n"/>
-      <c r="AL52" s="4" t="n"/>
-      <c r="AM52" s="4" t="n"/>
-      <c r="AN52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="X53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AB53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AF53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AH53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AI53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AJ53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AK53" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN53" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="4" t="n"/>
+      <c r="L53" s="4" t="n"/>
+      <c r="M53" s="4" t="n"/>
+      <c r="N53" s="4" t="n"/>
+      <c r="O53" s="4" t="n"/>
+      <c r="P53" s="4" t="n"/>
+      <c r="Q53" s="4" t="n"/>
+      <c r="R53" s="4" t="n"/>
+      <c r="S53" s="4" t="n"/>
+      <c r="T53" s="4" t="n"/>
+      <c r="U53" s="4" t="n"/>
+      <c r="V53" s="4" t="n"/>
+      <c r="W53" s="4" t="n"/>
+      <c r="X53" s="4" t="n"/>
+      <c r="Y53" s="4" t="n"/>
+      <c r="Z53" s="4" t="n"/>
+      <c r="AA53" s="4" t="n"/>
+      <c r="AB53" s="4" t="n"/>
+      <c r="AC53" s="4" t="n"/>
+      <c r="AD53" s="4" t="n"/>
+      <c r="AE53" s="4" t="n"/>
+      <c r="AF53" s="4" t="n"/>
+      <c r="AG53" s="4" t="n"/>
+      <c r="AH53" s="4" t="n"/>
+      <c r="AI53" s="4" t="n"/>
+      <c r="AJ53" s="4" t="n"/>
+      <c r="AK53" s="4" t="n"/>
+      <c r="AL53" s="4" t="n"/>
+      <c r="AM53" s="4" t="n"/>
+      <c r="AN53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>FTE</t>
+          <t>Headcount</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
@@ -6804,40 +6824,40 @@
         <v>2</v>
       </c>
       <c r="Z54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AB54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AC54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AD54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AE54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AF54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AG54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AH54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AI54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AJ54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AK54" s="4" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="AL54" s="4" t="n">
         <v>2</v>
@@ -6846,6 +6866,130 @@
         <v>2</v>
       </c>
       <c r="AN54" s="4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="W55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="X55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AA55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AB55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AC55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AD55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AE55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AF55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AG55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AH55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AI55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AJ55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AK55" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="AL55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN55" s="4" t="n">
         <v>2.25</v>
       </c>
     </row>
@@ -6895,7 +7039,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="C2" t="n">
         <v>1500</v>
@@ -6911,13 +7055,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="C3" t="n">
-        <v>375</v>
+        <v>575</v>
       </c>
       <c r="D3" t="n">
-        <v>1241.67</v>
+        <v>1441.67</v>
       </c>
     </row>
     <row r="4">
@@ -6927,13 +7071,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="C4" t="n">
-        <v>1125</v>
+        <v>925</v>
       </c>
       <c r="D4" t="n">
-        <v>1458.33</v>
+        <v>1258.33</v>
       </c>
     </row>
     <row r="5">
@@ -6975,13 +7119,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1979.92</v>
+        <v>8479.92</v>
       </c>
       <c r="C7" t="n">
-        <v>11825.53</v>
+        <v>18925.53</v>
       </c>
       <c r="D7" t="n">
-        <v>20567.68</v>
+        <v>27838.68</v>
       </c>
     </row>
     <row r="8">
@@ -6991,13 +7135,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1979.92</v>
+        <v>8929.92</v>
       </c>
       <c r="C8" t="n">
-        <v>32950.53</v>
+        <v>39850.53</v>
       </c>
       <c r="D8" t="n">
-        <v>42026.01</v>
+        <v>49097.01</v>
       </c>
     </row>
     <row r="9">
@@ -7026,7 +7170,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>790</v>
+        <v>619</v>
       </c>
       <c r="D10" t="n">
         <v>671</v>
@@ -7042,7 +7186,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>22456.67</v>
+        <v>22285.67</v>
       </c>
       <c r="D11" t="n">
         <v>28337.67</v>
@@ -7055,13 +7199,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1979.92</v>
+        <v>8929.92</v>
       </c>
       <c r="C12" t="n">
-        <v>10493.87</v>
+        <v>17564.87</v>
       </c>
       <c r="D12" t="n">
-        <v>13688.34</v>
+        <v>20759.34</v>
       </c>
     </row>
     <row r="13">
@@ -7071,13 +7215,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
       <c r="C13" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
       <c r="D13" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="14">
@@ -7087,13 +7231,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-4020.08</v>
+        <v>-5070.08</v>
       </c>
       <c r="C14" t="n">
-        <v>4493.87</v>
+        <v>3564.87</v>
       </c>
       <c r="D14" t="n">
-        <v>7688.34</v>
+        <v>6759.34</v>
       </c>
     </row>
     <row r="15">
@@ -7103,13 +7247,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1979.92</v>
+        <v>8929.92</v>
       </c>
       <c r="C15" t="n">
-        <v>10493.87</v>
+        <v>17564.87</v>
       </c>
       <c r="D15" t="n">
-        <v>13688.34</v>
+        <v>20759.34</v>
       </c>
     </row>
   </sheetData>
@@ -7123,7 +7267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN54"/>
+  <dimension ref="A1:AN55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9518,7 +9662,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>0</v>
@@ -9614,7 +9758,7 @@
         <v>0</v>
       </c>
       <c r="AL22" s="4" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="AM22" s="4" t="n">
         <v>1200</v>
@@ -9766,7 +9910,7 @@
         <v>71.55</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>373.23</v>
+        <v>573.23</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>74.08</v>
@@ -9862,7 +10006,7 @@
         <v>952.5700000000001</v>
       </c>
       <c r="AL24" s="4" t="n">
-        <v>1189.57</v>
+        <v>1389.57</v>
       </c>
       <c r="AM24" s="4" t="n">
         <v>4053.07</v>
@@ -9890,7 +10034,7 @@
         <v>-56.58</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>-353.27</v>
+        <v>-553.27</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>-54.12</v>
@@ -9986,7 +10130,7 @@
         <v>13771.33</v>
       </c>
       <c r="AL25" s="4" t="n">
-        <v>-620.08</v>
+        <v>-820.08</v>
       </c>
       <c r="AM25" s="4" t="n">
         <v>32710.23</v>
@@ -10668,40 +10812,40 @@
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>128</v>
+        <v>240</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>112</v>
+        <v>210</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>96</v>
+        <v>180</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>72</v>
+        <v>135</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>104</v>
+        <v>195</v>
       </c>
       <c r="N32" s="4" t="n">
         <v>840</v>
@@ -10776,7 +10920,7 @@
         <v>1560</v>
       </c>
       <c r="AL32" s="4" t="n">
-        <v>800</v>
+        <v>1500</v>
       </c>
       <c r="AM32" s="4" t="n">
         <v>5250</v>
@@ -11784,40 +11928,40 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>-481.27</v>
+        <v>-593.27</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>-585.71</v>
+        <v>-683.71</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>-271.23</v>
+        <v>-341.23</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>-607.58</v>
+        <v>-635.58</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>-584.27</v>
+        <v>-868.27</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-261.12</v>
+        <v>-324.12</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-241.27</v>
+        <v>-290.27</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>-201.64</v>
+        <v>-236.64</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>-193.95</v>
+        <v>-221.95</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>-186.15</v>
+        <v>-207.15</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>-137.32</v>
+        <v>-158.32</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>-268.57</v>
+        <v>-359.57</v>
       </c>
       <c r="N41" s="4" t="n">
         <v>-1622.11</v>
@@ -11892,7 +12036,7 @@
         <v>325.03</v>
       </c>
       <c r="AL41" s="4" t="n">
-        <v>-4020.08</v>
+        <v>-4920.08</v>
       </c>
       <c r="AM41" s="4" t="n">
         <v>21199.24</v>
@@ -11917,40 +12061,40 @@
         <v>0</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="I42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="J42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="O42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="P42" s="4" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="Q42" s="4" t="n">
         <v>41.67</v>
@@ -12016,10 +12160,10 @@
         <v>145.83</v>
       </c>
       <c r="AL42" s="4" t="n">
-        <v>0</v>
+        <v>150.03</v>
       </c>
       <c r="AM42" s="4" t="n">
-        <v>375.03</v>
+        <v>425.04</v>
       </c>
       <c r="AN42" s="4" t="n">
         <v>1726.35</v>
@@ -12032,49 +12176,49 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>-481.27</v>
+        <v>-593.27</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>-585.71</v>
+        <v>-683.71</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>-271.23</v>
+        <v>-341.23</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>-607.58</v>
+        <v>-652.24</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>-584.27</v>
+        <v>-884.9400000000001</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>-261.12</v>
+        <v>-340.79</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>-241.27</v>
+        <v>-306.93</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>-201.64</v>
+        <v>-253.31</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>-193.95</v>
+        <v>-238.62</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>-186.15</v>
+        <v>-223.82</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>-137.32</v>
+        <v>-174.98</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>-268.57</v>
+        <v>-376.24</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>-1622.11</v>
+        <v>-1638.77</v>
       </c>
       <c r="O43" s="4" t="n">
-        <v>80.16</v>
+        <v>63.5</v>
       </c>
       <c r="P43" s="4" t="n">
-        <v>944.47</v>
+        <v>927.8099999999999</v>
       </c>
       <c r="Q43" s="4" t="n">
         <v>235.46</v>
@@ -12140,10 +12284,10 @@
         <v>179.19</v>
       </c>
       <c r="AL43" s="4" t="n">
-        <v>-4020.08</v>
+        <v>-5070.08</v>
       </c>
       <c r="AM43" s="4" t="n">
-        <v>20824.23</v>
+        <v>20774.25</v>
       </c>
       <c r="AN43" s="4" t="n">
         <v>-17496.12</v>
@@ -12459,7 +12603,7 @@
         <v>0</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F47" s="4" t="n">
         <v>0</v>
@@ -12495,7 +12639,7 @@
         <v>0</v>
       </c>
       <c r="Q47" s="4" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="R47" s="4" t="n">
         <v>0</v>
@@ -12558,10 +12702,10 @@
         <v>0</v>
       </c>
       <c r="AL47" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="AM47" s="4" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="AN47" s="4" t="n">
         <v>3750</v>
@@ -12673,7 +12817,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>2979</v>
+        <v>2808</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -12688,555 +12832,555 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>2979</v>
+        <v>2808</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Total payments</t>
+          <t>Equity investment received</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
-        <v>481.27</v>
+        <v>0</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>585.71</v>
+        <v>3000</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>286.2</v>
+        <v>8000</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>622.55</v>
+        <v>0</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>604.23</v>
+        <v>0</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>281.08</v>
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="n">
-        <v>266.22</v>
+        <v>0</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>276.58</v>
+        <v>0</v>
       </c>
       <c r="J49" s="4" t="n">
-        <v>268.89</v>
+        <v>0</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>261.09</v>
+        <v>0</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>262.25</v>
+        <v>0</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>393.5</v>
+        <v>0</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>1816.99</v>
+        <v>0</v>
       </c>
       <c r="O49" s="4" t="n">
-        <v>1856.32</v>
+        <v>0</v>
       </c>
       <c r="P49" s="4" t="n">
-        <v>1056.97</v>
+        <v>0</v>
       </c>
       <c r="Q49" s="4" t="n">
-        <v>3229.31</v>
+        <v>0</v>
       </c>
       <c r="R49" s="4" t="n">
-        <v>1838.07</v>
+        <v>0</v>
       </c>
       <c r="S49" s="4" t="n">
-        <v>1089.57</v>
+        <v>0</v>
       </c>
       <c r="T49" s="4" t="n">
-        <v>990.28</v>
+        <v>0</v>
       </c>
       <c r="U49" s="4" t="n">
-        <v>889.2</v>
+        <v>0</v>
       </c>
       <c r="V49" s="4" t="n">
-        <v>840.17</v>
+        <v>0</v>
       </c>
       <c r="W49" s="4" t="n">
-        <v>788.8200000000001</v>
+        <v>0</v>
       </c>
       <c r="X49" s="4" t="n">
-        <v>790.48</v>
+        <v>0</v>
       </c>
       <c r="Y49" s="4" t="n">
-        <v>1877.9</v>
+        <v>0</v>
       </c>
       <c r="Z49" s="4" t="n">
-        <v>14478.45</v>
+        <v>0</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>15969.43</v>
+        <v>0</v>
       </c>
       <c r="AB49" s="4" t="n">
-        <v>13653.84</v>
+        <v>0</v>
       </c>
       <c r="AC49" s="4" t="n">
-        <v>14738.97</v>
+        <v>0</v>
       </c>
       <c r="AD49" s="4" t="n">
-        <v>14005.75</v>
+        <v>0</v>
       </c>
       <c r="AE49" s="4" t="n">
-        <v>14072.71</v>
+        <v>0</v>
       </c>
       <c r="AF49" s="4" t="n">
-        <v>14754</v>
+        <v>0</v>
       </c>
       <c r="AG49" s="4" t="n">
-        <v>13326.38</v>
+        <v>0</v>
       </c>
       <c r="AH49" s="4" t="n">
-        <v>13215.53</v>
+        <v>0</v>
       </c>
       <c r="AI49" s="4" t="n">
-        <v>16079.59</v>
+        <v>0</v>
       </c>
       <c r="AJ49" s="4" t="n">
-        <v>13106.18</v>
+        <v>0</v>
       </c>
       <c r="AK49" s="4" t="n">
-        <v>14398.87</v>
+        <v>0</v>
       </c>
       <c r="AL49" s="4" t="n">
-        <v>4589.57</v>
+        <v>11000</v>
       </c>
       <c r="AM49" s="4" t="n">
-        <v>17064.08</v>
+        <v>0</v>
       </c>
       <c r="AN49" s="4" t="n">
-        <v>171799.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Net cash flow</t>
+          <t>Total payments</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>-481.27</v>
+        <v>593.27</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>-585.71</v>
+        <v>683.71</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>-271.23</v>
+        <v>356.2</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>-607.58</v>
+        <v>1250.55</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>-584.27</v>
+        <v>888.23</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>-261.12</v>
+        <v>344.08</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>-241.27</v>
+        <v>315.22</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>-201.64</v>
+        <v>311.58</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>-193.95</v>
+        <v>296.89</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>-186.15</v>
+        <v>282.09</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>-137.32</v>
+        <v>283.25</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>-268.57</v>
+        <v>484.5</v>
       </c>
       <c r="N50" s="4" t="n">
-        <v>-1622.11</v>
+        <v>1816.99</v>
       </c>
       <c r="O50" s="4" t="n">
-        <v>18413.5</v>
+        <v>1856.32</v>
       </c>
       <c r="P50" s="4" t="n">
-        <v>-722.1900000000001</v>
+        <v>1056.97</v>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>-2889.54</v>
+        <v>2629.31</v>
       </c>
       <c r="R50" s="4" t="n">
-        <v>18571.65</v>
+        <v>1838.07</v>
       </c>
       <c r="S50" s="4" t="n">
-        <v>-619.88</v>
+        <v>1089.57</v>
       </c>
       <c r="T50" s="4" t="n">
-        <v>-515.6</v>
+        <v>990.28</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>-409.53</v>
+        <v>889.2</v>
       </c>
       <c r="V50" s="4" t="n">
-        <v>-310.51</v>
+        <v>840.17</v>
       </c>
       <c r="W50" s="4" t="n">
-        <v>-264.15</v>
+        <v>788.8200000000001</v>
       </c>
       <c r="X50" s="4" t="n">
-        <v>-265.81</v>
+        <v>790.48</v>
       </c>
       <c r="Y50" s="4" t="n">
-        <v>-1333.27</v>
+        <v>1877.9</v>
       </c>
       <c r="Z50" s="4" t="n">
-        <v>30181.04</v>
+        <v>14478.45</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>20814.9</v>
+        <v>15969.43</v>
       </c>
       <c r="AB50" s="4" t="n">
-        <v>-12774.61</v>
+        <v>13653.84</v>
       </c>
       <c r="AC50" s="4" t="n">
-        <v>16195.24</v>
+        <v>14738.97</v>
       </c>
       <c r="AD50" s="4" t="n">
-        <v>7028.35</v>
+        <v>14005.75</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>-13058.66</v>
+        <v>14072.71</v>
       </c>
       <c r="AF50" s="4" t="n">
-        <v>18330</v>
+        <v>14754</v>
       </c>
       <c r="AG50" s="4" t="n">
-        <v>-12237.39</v>
+        <v>13326.38</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>-12081.54</v>
+        <v>13215.53</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>-14950.59</v>
+        <v>15908.59</v>
       </c>
       <c r="AJ50" s="4" t="n">
-        <v>-11937.17</v>
+        <v>13106.18</v>
       </c>
       <c r="AK50" s="4" t="n">
-        <v>-13174.97</v>
+        <v>14398.87</v>
       </c>
       <c r="AL50" s="4" t="n">
-        <v>-4020.08</v>
+        <v>6089.57</v>
       </c>
       <c r="AM50" s="4" t="n">
-        <v>28032.56</v>
+        <v>16464.08</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>2334.6</v>
+        <v>171628.7</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Net cash flow</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n">
+        <v>-593.27</v>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>2316.29</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>7658.77</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>-1235.58</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>-868.27</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>-324.12</v>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>-290.27</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>-236.64</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>-221.95</v>
+      </c>
+      <c r="K51" s="4" t="n">
+        <v>-207.15</v>
+      </c>
+      <c r="L51" s="4" t="n">
+        <v>-158.32</v>
+      </c>
+      <c r="M51" s="4" t="n">
+        <v>-359.57</v>
+      </c>
+      <c r="N51" s="4" t="n">
+        <v>-1622.11</v>
+      </c>
+      <c r="O51" s="4" t="n">
+        <v>18413.5</v>
+      </c>
+      <c r="P51" s="4" t="n">
+        <v>-722.1900000000001</v>
+      </c>
+      <c r="Q51" s="4" t="n">
+        <v>-2289.54</v>
+      </c>
+      <c r="R51" s="4" t="n">
+        <v>18571.65</v>
+      </c>
+      <c r="S51" s="4" t="n">
+        <v>-619.88</v>
+      </c>
+      <c r="T51" s="4" t="n">
+        <v>-515.6</v>
+      </c>
+      <c r="U51" s="4" t="n">
+        <v>-409.53</v>
+      </c>
+      <c r="V51" s="4" t="n">
+        <v>-310.51</v>
+      </c>
+      <c r="W51" s="4" t="n">
+        <v>-264.15</v>
+      </c>
+      <c r="X51" s="4" t="n">
+        <v>-265.81</v>
+      </c>
+      <c r="Y51" s="4" t="n">
+        <v>-1333.27</v>
+      </c>
+      <c r="Z51" s="4" t="n">
+        <v>30181.04</v>
+      </c>
+      <c r="AA51" s="4" t="n">
+        <v>20814.9</v>
+      </c>
+      <c r="AB51" s="4" t="n">
+        <v>-12774.61</v>
+      </c>
+      <c r="AC51" s="4" t="n">
+        <v>16195.24</v>
+      </c>
+      <c r="AD51" s="4" t="n">
+        <v>7028.35</v>
+      </c>
+      <c r="AE51" s="4" t="n">
+        <v>-13058.66</v>
+      </c>
+      <c r="AF51" s="4" t="n">
+        <v>18330</v>
+      </c>
+      <c r="AG51" s="4" t="n">
+        <v>-12237.39</v>
+      </c>
+      <c r="AH51" s="4" t="n">
+        <v>-12081.54</v>
+      </c>
+      <c r="AI51" s="4" t="n">
+        <v>-14779.59</v>
+      </c>
+      <c r="AJ51" s="4" t="n">
+        <v>-11937.17</v>
+      </c>
+      <c r="AK51" s="4" t="n">
+        <v>-13174.97</v>
+      </c>
+      <c r="AL51" s="4" t="n">
+        <v>5479.92</v>
+      </c>
+      <c r="AM51" s="4" t="n">
+        <v>28632.56</v>
+      </c>
+      <c r="AN51" s="4" t="n">
+        <v>2505.6</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Closing cash</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n">
-        <v>5518.73</v>
-      </c>
-      <c r="C51" s="4" t="n">
-        <v>4933.02</v>
-      </c>
-      <c r="D51" s="4" t="n">
-        <v>4661.79</v>
-      </c>
-      <c r="E51" s="4" t="n">
-        <v>4054.21</v>
-      </c>
-      <c r="F51" s="4" t="n">
-        <v>3469.94</v>
-      </c>
-      <c r="G51" s="4" t="n">
-        <v>3208.82</v>
-      </c>
-      <c r="H51" s="4" t="n">
-        <v>2967.55</v>
-      </c>
-      <c r="I51" s="4" t="n">
-        <v>2765.91</v>
-      </c>
-      <c r="J51" s="4" t="n">
-        <v>2571.96</v>
-      </c>
-      <c r="K51" s="4" t="n">
-        <v>2385.81</v>
-      </c>
-      <c r="L51" s="4" t="n">
-        <v>2248.49</v>
-      </c>
-      <c r="M51" s="4" t="n">
-        <v>1979.92</v>
-      </c>
-      <c r="N51" s="4" t="n">
-        <v>357.82</v>
-      </c>
-      <c r="O51" s="4" t="n">
-        <v>18771.31</v>
-      </c>
-      <c r="P51" s="4" t="n">
-        <v>18049.12</v>
-      </c>
-      <c r="Q51" s="4" t="n">
-        <v>15159.58</v>
-      </c>
-      <c r="R51" s="4" t="n">
-        <v>33731.23</v>
-      </c>
-      <c r="S51" s="4" t="n">
-        <v>33111.35</v>
-      </c>
-      <c r="T51" s="4" t="n">
-        <v>32595.75</v>
-      </c>
-      <c r="U51" s="4" t="n">
-        <v>32186.22</v>
-      </c>
-      <c r="V51" s="4" t="n">
-        <v>31875.71</v>
-      </c>
-      <c r="W51" s="4" t="n">
-        <v>31611.57</v>
-      </c>
-      <c r="X51" s="4" t="n">
-        <v>31345.76</v>
-      </c>
-      <c r="Y51" s="4" t="n">
-        <v>30012.49</v>
-      </c>
-      <c r="Z51" s="4" t="n">
-        <v>60193.53</v>
-      </c>
-      <c r="AA51" s="4" t="n">
-        <v>81008.42999999999</v>
-      </c>
-      <c r="AB51" s="4" t="n">
-        <v>68233.82000000001</v>
-      </c>
-      <c r="AC51" s="4" t="n">
-        <v>84429.06</v>
-      </c>
-      <c r="AD51" s="4" t="n">
-        <v>91457.41</v>
-      </c>
-      <c r="AE51" s="4" t="n">
-        <v>78398.75</v>
-      </c>
-      <c r="AF51" s="4" t="n">
-        <v>96728.75</v>
-      </c>
-      <c r="AG51" s="4" t="n">
-        <v>84491.36</v>
-      </c>
-      <c r="AH51" s="4" t="n">
-        <v>72409.82000000001</v>
-      </c>
-      <c r="AI51" s="4" t="n">
-        <v>57459.23</v>
-      </c>
-      <c r="AJ51" s="4" t="n">
-        <v>45522.06</v>
-      </c>
-      <c r="AK51" s="4" t="n">
-        <v>32347.09</v>
-      </c>
-      <c r="AL51" s="4" t="n">
-        <v>1979.92</v>
-      </c>
-      <c r="AM51" s="4" t="n">
-        <v>30012.49</v>
-      </c>
-      <c r="AN51" s="4" t="n">
-        <v>32347.09</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="B52" s="4" t="n">
+        <v>2406.73</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>4723.02</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>12381.79</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>11146.21</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>10277.94</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>9953.82</v>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>9663.549999999999</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>9426.91</v>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>9204.959999999999</v>
+      </c>
+      <c r="K52" s="4" t="n">
+        <v>8997.809999999999</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>8839.49</v>
+      </c>
+      <c r="M52" s="4" t="n">
+        <v>8479.92</v>
+      </c>
+      <c r="N52" s="4" t="n">
+        <v>6857.82</v>
+      </c>
+      <c r="O52" s="4" t="n">
+        <v>25271.31</v>
+      </c>
+      <c r="P52" s="4" t="n">
+        <v>24549.12</v>
+      </c>
+      <c r="Q52" s="4" t="n">
+        <v>22259.58</v>
+      </c>
+      <c r="R52" s="4" t="n">
+        <v>40831.23</v>
+      </c>
+      <c r="S52" s="4" t="n">
+        <v>40211.35</v>
+      </c>
+      <c r="T52" s="4" t="n">
+        <v>39695.75</v>
+      </c>
+      <c r="U52" s="4" t="n">
+        <v>39286.22</v>
+      </c>
+      <c r="V52" s="4" t="n">
+        <v>38975.71</v>
+      </c>
+      <c r="W52" s="4" t="n">
+        <v>38711.57</v>
+      </c>
+      <c r="X52" s="4" t="n">
+        <v>38445.76</v>
+      </c>
+      <c r="Y52" s="4" t="n">
+        <v>37112.49</v>
+      </c>
+      <c r="Z52" s="4" t="n">
+        <v>67293.53</v>
+      </c>
+      <c r="AA52" s="4" t="n">
+        <v>88108.42999999999</v>
+      </c>
+      <c r="AB52" s="4" t="n">
+        <v>75333.82000000001</v>
+      </c>
+      <c r="AC52" s="4" t="n">
+        <v>91529.06</v>
+      </c>
+      <c r="AD52" s="4" t="n">
+        <v>98557.41</v>
+      </c>
+      <c r="AE52" s="4" t="n">
+        <v>85498.75</v>
+      </c>
+      <c r="AF52" s="4" t="n">
+        <v>103828.75</v>
+      </c>
+      <c r="AG52" s="4" t="n">
+        <v>91591.36</v>
+      </c>
+      <c r="AH52" s="4" t="n">
+        <v>79509.82000000001</v>
+      </c>
+      <c r="AI52" s="4" t="n">
+        <v>64730.23</v>
+      </c>
+      <c r="AJ52" s="4" t="n">
+        <v>52793.06</v>
+      </c>
+      <c r="AK52" s="4" t="n">
+        <v>39618.09</v>
+      </c>
+      <c r="AL52" s="4" t="n">
+        <v>8479.92</v>
+      </c>
+      <c r="AM52" s="4" t="n">
+        <v>37112.49</v>
+      </c>
+      <c r="AN52" s="4" t="n">
+        <v>39618.09</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>TEAM</t>
         </is>
       </c>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
-      <c r="K52" s="4" t="n"/>
-      <c r="L52" s="4" t="n"/>
-      <c r="M52" s="4" t="n"/>
-      <c r="N52" s="4" t="n"/>
-      <c r="O52" s="4" t="n"/>
-      <c r="P52" s="4" t="n"/>
-      <c r="Q52" s="4" t="n"/>
-      <c r="R52" s="4" t="n"/>
-      <c r="S52" s="4" t="n"/>
-      <c r="T52" s="4" t="n"/>
-      <c r="U52" s="4" t="n"/>
-      <c r="V52" s="4" t="n"/>
-      <c r="W52" s="4" t="n"/>
-      <c r="X52" s="4" t="n"/>
-      <c r="Y52" s="4" t="n"/>
-      <c r="Z52" s="4" t="n"/>
-      <c r="AA52" s="4" t="n"/>
-      <c r="AB52" s="4" t="n"/>
-      <c r="AC52" s="4" t="n"/>
-      <c r="AD52" s="4" t="n"/>
-      <c r="AE52" s="4" t="n"/>
-      <c r="AF52" s="4" t="n"/>
-      <c r="AG52" s="4" t="n"/>
-      <c r="AH52" s="4" t="n"/>
-      <c r="AI52" s="4" t="n"/>
-      <c r="AJ52" s="4" t="n"/>
-      <c r="AK52" s="4" t="n"/>
-      <c r="AL52" s="4" t="n"/>
-      <c r="AM52" s="4" t="n"/>
-      <c r="AN52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Headcount</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="J53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="M53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="R53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="S53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="T53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="U53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="V53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="W53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="X53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z53" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AC53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AD53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AE53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AF53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AH53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AI53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AJ53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AK53" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="AL53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM53" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN53" s="4" t="n">
-        <v>6</v>
-      </c>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
+      <c r="J53" s="4" t="n"/>
+      <c r="K53" s="4" t="n"/>
+      <c r="L53" s="4" t="n"/>
+      <c r="M53" s="4" t="n"/>
+      <c r="N53" s="4" t="n"/>
+      <c r="O53" s="4" t="n"/>
+      <c r="P53" s="4" t="n"/>
+      <c r="Q53" s="4" t="n"/>
+      <c r="R53" s="4" t="n"/>
+      <c r="S53" s="4" t="n"/>
+      <c r="T53" s="4" t="n"/>
+      <c r="U53" s="4" t="n"/>
+      <c r="V53" s="4" t="n"/>
+      <c r="W53" s="4" t="n"/>
+      <c r="X53" s="4" t="n"/>
+      <c r="Y53" s="4" t="n"/>
+      <c r="Z53" s="4" t="n"/>
+      <c r="AA53" s="4" t="n"/>
+      <c r="AB53" s="4" t="n"/>
+      <c r="AC53" s="4" t="n"/>
+      <c r="AD53" s="4" t="n"/>
+      <c r="AE53" s="4" t="n"/>
+      <c r="AF53" s="4" t="n"/>
+      <c r="AG53" s="4" t="n"/>
+      <c r="AH53" s="4" t="n"/>
+      <c r="AI53" s="4" t="n"/>
+      <c r="AJ53" s="4" t="n"/>
+      <c r="AK53" s="4" t="n"/>
+      <c r="AL53" s="4" t="n"/>
+      <c r="AM53" s="4" t="n"/>
+      <c r="AN53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>FTE</t>
+          <t>Headcount</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
@@ -13312,40 +13456,40 @@
         <v>2</v>
       </c>
       <c r="Z54" s="4" t="n">
-        <v>3.25</v>
+        <v>4</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AB54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AC54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AD54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AE54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AF54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AG54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AH54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AI54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AJ54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AK54" s="4" t="n">
-        <v>5.25</v>
+        <v>6</v>
       </c>
       <c r="AL54" s="4" t="n">
         <v>2</v>
@@ -13354,6 +13498,130 @@
         <v>2</v>
       </c>
       <c r="AN54" s="4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>FTE</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="R55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="T55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="U55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="W55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="X55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z55" s="4" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="AA55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AB55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AC55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AD55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AE55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AF55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AG55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AH55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AI55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AJ55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AK55" s="4" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="AL55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM55" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN55" s="4" t="n">
         <v>5.25</v>
       </c>
     </row>
@@ -13403,7 +13671,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="C2" t="n">
         <v>1500</v>
@@ -13419,13 +13687,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="C3" t="n">
-        <v>375</v>
+        <v>575</v>
       </c>
       <c r="D3" t="n">
-        <v>2101.39</v>
+        <v>2301.39</v>
       </c>
     </row>
     <row r="4">
@@ -13435,13 +13703,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="C4" t="n">
-        <v>1125</v>
+        <v>925</v>
       </c>
       <c r="D4" t="n">
-        <v>3148.61</v>
+        <v>2948.61</v>
       </c>
     </row>
     <row r="5">
@@ -13483,13 +13751,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1979.92</v>
+        <v>8479.92</v>
       </c>
       <c r="C7" t="n">
-        <v>30012.49</v>
+        <v>37112.49</v>
       </c>
       <c r="D7" t="n">
-        <v>32347.09</v>
+        <v>39618.09</v>
       </c>
     </row>
     <row r="8">
@@ -13499,13 +13767,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1979.92</v>
+        <v>8929.92</v>
       </c>
       <c r="C8" t="n">
-        <v>75137.49000000001</v>
+        <v>82037.49000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>79495.7</v>
+        <v>86566.7</v>
       </c>
     </row>
     <row r="9">
@@ -13534,7 +13802,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>2979</v>
+        <v>2808</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -13550,7 +13818,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>55312.33</v>
+        <v>55141.33</v>
       </c>
       <c r="D11" t="n">
         <v>77166.67</v>
@@ -13563,13 +13831,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1979.92</v>
+        <v>8929.92</v>
       </c>
       <c r="C12" t="n">
-        <v>19825.16</v>
+        <v>26896.16</v>
       </c>
       <c r="D12" t="n">
-        <v>2329.03</v>
+        <v>9400.030000000001</v>
       </c>
     </row>
     <row r="13">
@@ -13579,13 +13847,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
       <c r="C13" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
       <c r="D13" t="n">
-        <v>6000</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="14">
@@ -13595,13 +13863,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-4020.08</v>
+        <v>-5070.08</v>
       </c>
       <c r="C14" t="n">
-        <v>13825.16</v>
+        <v>12896.16</v>
       </c>
       <c r="D14" t="n">
-        <v>-3670.97</v>
+        <v>-4599.97</v>
       </c>
     </row>
     <row r="15">
@@ -13611,13 +13879,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1979.92</v>
+        <v>8929.92</v>
       </c>
       <c r="C15" t="n">
-        <v>19825.16</v>
+        <v>26896.16</v>
       </c>
       <c r="D15" t="n">
-        <v>2329.03</v>
+        <v>9400.030000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business plan v6: sole founder, investment conditional on pilot + LOI
- Yusuf Quadri as sole founder; co-founder removed; engineering led by
  wider team with paid Software Engineer role from Year 3
- £3,000 founder capital up front; £11,000 equity (friends & family,
  Nigerian company) released after successful pilot and signed LOI
- Lean pre-pilot spending profile; downside case now models pilot
  failure with no investment
- Research evidence pack section referencing the submission folder

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146q3FtAYmgQ1rtNsNNpdiD
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
@@ -573,7 +573,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Founders' opening capital (£)</t>
+          <t>Founder's opening capital (£)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -583,7 +583,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Friends &amp; family equity (£, Oct 2026)</t>
+          <t>Friends &amp; family equity (£, Apr 2027, after pilot + LOI)</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -593,7 +593,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nigerian company equity (£, Nov 2026)</t>
+          <t>Nigerian company equity (£, Apr 2027, after pilot + LOI)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -3030,7 +3030,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>0</v>
@@ -3126,7 +3126,7 @@
         <v>0</v>
       </c>
       <c r="AL22" s="4" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="AM22" s="4" t="n">
         <v>600</v>
@@ -3278,7 +3278,7 @@
         <v>71.55</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>573.23</v>
+        <v>373.23</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>74.08</v>
@@ -3374,7 +3374,7 @@
         <v>463.22</v>
       </c>
       <c r="AL24" s="4" t="n">
-        <v>1389.57</v>
+        <v>1189.57</v>
       </c>
       <c r="AM24" s="4" t="n">
         <v>2670.96</v>
@@ -3402,7 +3402,7 @@
         <v>-56.58</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>-553.27</v>
+        <v>-353.27</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>-54.12</v>
@@ -3498,7 +3498,7 @@
         <v>4714.41</v>
       </c>
       <c r="AL25" s="4" t="n">
-        <v>-820.08</v>
+        <v>-620.08</v>
       </c>
       <c r="AM25" s="4" t="n">
         <v>19439.96</v>
@@ -3632,40 +3632,40 @@
         <v>0</v>
       </c>
       <c r="Z27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AD27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AE27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AF27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AG27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AI27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AK27" s="4" t="n">
-        <v>2333.33</v>
+        <v>2541.67</v>
       </c>
       <c r="AL27" s="4" t="n">
         <v>0</v>
@@ -3674,7 +3674,7 @@
         <v>0</v>
       </c>
       <c r="AN27" s="4" t="n">
-        <v>27999.96</v>
+        <v>30500.04</v>
       </c>
     </row>
     <row r="28">
@@ -3880,40 +3880,40 @@
         <v>0</v>
       </c>
       <c r="Z29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AD29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AE29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AF29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AG29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AI29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AK29" s="4" t="n">
-        <v>70</v>
+        <v>76.25</v>
       </c>
       <c r="AL29" s="4" t="n">
         <v>0</v>
@@ -3922,7 +3922,7 @@
         <v>0</v>
       </c>
       <c r="AN29" s="4" t="n">
-        <v>840</v>
+        <v>915</v>
       </c>
     </row>
     <row r="30">
@@ -4004,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="Z30" s="4" t="n">
-        <v>210</v>
+        <v>420</v>
       </c>
       <c r="AA30" s="4" t="n">
         <v>0</v>
@@ -4046,7 +4046,7 @@
         <v>0</v>
       </c>
       <c r="AN30" s="4" t="n">
-        <v>210</v>
+        <v>420</v>
       </c>
     </row>
     <row r="31">
@@ -4128,40 +4128,40 @@
         <v>0</v>
       </c>
       <c r="Z31" s="4" t="n">
-        <v>2613.33</v>
+        <v>3037.92</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AD31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AE31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AF31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AG31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AI31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AK31" s="4" t="n">
-        <v>2403.33</v>
+        <v>2617.92</v>
       </c>
       <c r="AL31" s="4" t="n">
         <v>0</v>
@@ -4170,7 +4170,7 @@
         <v>0</v>
       </c>
       <c r="AN31" s="4" t="n">
-        <v>29049.96</v>
+        <v>31835.04</v>
       </c>
     </row>
     <row r="32">
@@ -4180,40 +4180,40 @@
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>240</v>
+        <v>75</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>210</v>
+        <v>75</v>
       </c>
       <c r="D32" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I32" s="4" t="n">
         <v>150</v>
       </c>
-      <c r="E32" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="G32" s="4" t="n">
-        <v>135</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="I32" s="4" t="n">
-        <v>75</v>
-      </c>
       <c r="J32" s="4" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>45</v>
+        <v>225</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>195</v>
+        <v>450</v>
       </c>
       <c r="N32" s="4" t="n">
         <v>560</v>
@@ -4927,28 +4927,28 @@
         <v>52</v>
       </c>
       <c r="C38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="D38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="4" t="n">
+      <c r="J38" s="4" t="n">
         <v>384</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K38" s="4" t="n">
         <v>0</v>
@@ -4969,22 +4969,22 @@
         <v>0</v>
       </c>
       <c r="Q38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" s="4" t="n">
         <v>384</v>
-      </c>
-      <c r="R38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V38" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0</v>
@@ -5005,22 +5005,22 @@
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH38" s="4" t="n">
         <v>384</v>
-      </c>
-      <c r="AD38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH38" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="AI38" s="4" t="n">
         <v>0</v>
@@ -5296,40 +5296,40 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>-593.27</v>
+        <v>-428.27</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>-683.71</v>
+        <v>-278.71</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>-341.23</v>
+        <v>-236.23</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>-635.58</v>
+        <v>-221.58</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>-868.27</v>
+        <v>-563.27</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-324.12</v>
+        <v>-234.12</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-290.27</v>
+        <v>-215.27</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>-236.64</v>
+        <v>-581.64</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>-221.95</v>
+        <v>-695.95</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>-207.15</v>
+        <v>-312.15</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>-158.32</v>
+        <v>-338.32</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>-359.57</v>
+        <v>-614.5700000000001</v>
       </c>
       <c r="N41" s="4" t="n">
         <v>-1341</v>
@@ -5341,7 +5341,7 @@
         <v>1066.2</v>
       </c>
       <c r="Q41" s="4" t="n">
-        <v>290.54</v>
+        <v>674.54</v>
       </c>
       <c r="R41" s="4" t="n">
         <v>997.67</v>
@@ -5356,7 +5356,7 @@
         <v>1295.88</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>1378.44</v>
+        <v>994.4400000000001</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>1412.48</v>
@@ -5368,49 +5368,49 @@
         <v>514.26</v>
       </c>
       <c r="Z41" s="4" t="n">
-        <v>-1335.85</v>
+        <v>-1760.43</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>-257.5</v>
+        <v>-472.09</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>41.29</v>
+        <v>-173.29</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>-736.85</v>
+        <v>-567.4400000000001</v>
       </c>
       <c r="AD41" s="4" t="n">
-        <v>-22.2</v>
+        <v>-236.78</v>
       </c>
       <c r="AE41" s="4" t="n">
-        <v>-288.7</v>
+        <v>-503.28</v>
       </c>
       <c r="AF41" s="4" t="n">
-        <v>621.3</v>
+        <v>406.72</v>
       </c>
       <c r="AG41" s="4" t="n">
-        <v>1340.64</v>
+        <v>1126.06</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>1441.44</v>
+        <v>842.86</v>
       </c>
       <c r="AI41" s="4" t="n">
-        <v>1494.59</v>
+        <v>1280.01</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>1536.74</v>
+        <v>1322.15</v>
       </c>
       <c r="AK41" s="4" t="n">
-        <v>897.25</v>
+        <v>682.66</v>
       </c>
       <c r="AL41" s="4" t="n">
-        <v>-4920.08</v>
+        <v>-4720.08</v>
       </c>
       <c r="AM41" s="4" t="n">
         <v>9678.940000000001</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>4732.15</v>
+        <v>1947.15</v>
       </c>
     </row>
     <row r="42">
@@ -5429,16 +5429,16 @@
         <v>0</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="I42" s="4" t="n">
         <v>16.67</v>
@@ -5528,7 +5528,7 @@
         <v>75</v>
       </c>
       <c r="AL42" s="4" t="n">
-        <v>150.03</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="AM42" s="4" t="n">
         <v>425.04</v>
@@ -5544,40 +5544,40 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>-593.27</v>
+        <v>-428.27</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>-683.71</v>
+        <v>-278.71</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>-341.23</v>
+        <v>-236.23</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>-652.24</v>
+        <v>-221.58</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>-884.9400000000001</v>
+        <v>-563.27</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>-340.79</v>
+        <v>-234.12</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>-306.93</v>
+        <v>-215.27</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>-253.31</v>
+        <v>-598.3099999999999</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>-238.62</v>
+        <v>-712.62</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>-223.82</v>
+        <v>-328.82</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>-174.98</v>
+        <v>-354.98</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>-376.24</v>
+        <v>-631.24</v>
       </c>
       <c r="N43" s="4" t="n">
         <v>-1357.66</v>
@@ -5589,7 +5589,7 @@
         <v>1049.53</v>
       </c>
       <c r="Q43" s="4" t="n">
-        <v>248.87</v>
+        <v>632.87</v>
       </c>
       <c r="R43" s="4" t="n">
         <v>956.01</v>
@@ -5604,7 +5604,7 @@
         <v>1254.21</v>
       </c>
       <c r="V43" s="4" t="n">
-        <v>1336.77</v>
+        <v>952.77</v>
       </c>
       <c r="W43" s="4" t="n">
         <v>1370.81</v>
@@ -5616,49 +5616,49 @@
         <v>472.6</v>
       </c>
       <c r="Z43" s="4" t="n">
-        <v>-1377.52</v>
+        <v>-1802.1</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>-332.5</v>
+        <v>-547.09</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>-33.71</v>
+        <v>-248.29</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>-811.85</v>
+        <v>-642.4400000000001</v>
       </c>
       <c r="AD43" s="4" t="n">
-        <v>-97.2</v>
+        <v>-311.78</v>
       </c>
       <c r="AE43" s="4" t="n">
-        <v>-363.7</v>
+        <v>-578.28</v>
       </c>
       <c r="AF43" s="4" t="n">
-        <v>546.3</v>
+        <v>331.72</v>
       </c>
       <c r="AG43" s="4" t="n">
-        <v>1265.64</v>
+        <v>1051.06</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>1366.44</v>
+        <v>767.86</v>
       </c>
       <c r="AI43" s="4" t="n">
-        <v>1419.59</v>
+        <v>1205.01</v>
       </c>
       <c r="AJ43" s="4" t="n">
-        <v>1461.74</v>
+        <v>1247.15</v>
       </c>
       <c r="AK43" s="4" t="n">
-        <v>822.25</v>
+        <v>607.66</v>
       </c>
       <c r="AL43" s="4" t="n">
-        <v>-5070.08</v>
+        <v>-4803.42</v>
       </c>
       <c r="AM43" s="4" t="n">
         <v>9253.940000000001</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>3865.48</v>
+        <v>1080.48</v>
       </c>
     </row>
     <row r="44">
@@ -5971,19 +5971,19 @@
         <v>0</v>
       </c>
       <c r="E47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4" t="n">
         <v>600</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J47" s="4" t="n">
         <v>0</v>
@@ -6185,7 +6185,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>619</v>
+        <v>657</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -6200,7 +6200,7 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>619</v>
+        <v>657</v>
       </c>
     </row>
     <row r="49">
@@ -6213,10 +6213,10 @@
         <v>0</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>0</v>
@@ -6231,7 +6231,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="J49" s="4" t="n">
         <v>0</v>
@@ -6334,40 +6334,40 @@
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>593.27</v>
+        <v>428.27</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>683.71</v>
+        <v>278.71</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>356.2</v>
+        <v>251.2</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>1250.55</v>
+        <v>236.55</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>888.23</v>
+        <v>583.23</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>344.08</v>
+        <v>254.08</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>315.22</v>
+        <v>240.22</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>311.58</v>
+        <v>1256.58</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>296.89</v>
+        <v>770.89</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>282.09</v>
+        <v>387.09</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>283.25</v>
+        <v>463.25</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>484.5</v>
+        <v>739.5</v>
       </c>
       <c r="N50" s="4" t="n">
         <v>1530.89</v>
@@ -6379,7 +6379,7 @@
         <v>865.3</v>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>2540.96</v>
+        <v>2156.96</v>
       </c>
       <c r="R50" s="4" t="n">
         <v>943.8</v>
@@ -6394,7 +6394,7 @@
         <v>710.5599999999999</v>
       </c>
       <c r="V50" s="4" t="n">
-        <v>677.99</v>
+        <v>1061.99</v>
       </c>
       <c r="W50" s="4" t="n">
         <v>643.95</v>
@@ -6406,49 +6406,49 @@
         <v>1552.14</v>
       </c>
       <c r="Z50" s="4" t="n">
-        <v>5173.8</v>
+        <v>5598.39</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>5335.38</v>
+        <v>5549.96</v>
       </c>
       <c r="AB50" s="4" t="n">
-        <v>3911.52</v>
+        <v>4126.11</v>
       </c>
       <c r="AC50" s="4" t="n">
-        <v>4689.67</v>
+        <v>4520.25</v>
       </c>
       <c r="AD50" s="4" t="n">
-        <v>4054.94</v>
+        <v>4269.53</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>4286.42</v>
+        <v>4501.01</v>
       </c>
       <c r="AF50" s="4" t="n">
-        <v>4436.39</v>
+        <v>4650.97</v>
       </c>
       <c r="AG50" s="4" t="n">
-        <v>3722.04</v>
+        <v>3936.63</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>3666.24</v>
+        <v>4264.82</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>4227.1</v>
+        <v>4479.69</v>
       </c>
       <c r="AJ50" s="4" t="n">
-        <v>3610.96</v>
+        <v>3825.54</v>
       </c>
       <c r="AK50" s="4" t="n">
-        <v>4280.39</v>
+        <v>4494.97</v>
       </c>
       <c r="AL50" s="4" t="n">
-        <v>6089.57</v>
+        <v>5889.57</v>
       </c>
       <c r="AM50" s="4" t="n">
         <v>13331.97</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>51394.85</v>
+        <v>54217.87</v>
       </c>
     </row>
     <row r="51">
@@ -6458,40 +6458,40 @@
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>-593.27</v>
+        <v>-428.27</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>2316.29</v>
+        <v>-278.71</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>7658.77</v>
+        <v>-236.23</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>-1235.58</v>
+        <v>-221.58</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>-868.27</v>
+        <v>-563.27</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>-324.12</v>
+        <v>-234.12</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>-290.27</v>
+        <v>-215.27</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>-236.64</v>
+        <v>9818.360000000001</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>-221.95</v>
+        <v>-695.95</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>-207.15</v>
+        <v>-312.15</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>-158.32</v>
+        <v>-338.32</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>-359.57</v>
+        <v>-614.5700000000001</v>
       </c>
       <c r="N51" s="4" t="n">
         <v>-1341</v>
@@ -6503,7 +6503,7 @@
         <v>-600.47</v>
       </c>
       <c r="Q51" s="4" t="n">
-        <v>-2276.13</v>
+        <v>-1892.13</v>
       </c>
       <c r="R51" s="4" t="n">
         <v>-668.99</v>
@@ -6518,7 +6518,7 @@
         <v>-370.79</v>
       </c>
       <c r="V51" s="4" t="n">
-        <v>-288.23</v>
+        <v>-672.23</v>
       </c>
       <c r="W51" s="4" t="n">
         <v>-254.19</v>
@@ -6530,49 +6530,49 @@
         <v>-1152.4</v>
       </c>
       <c r="Z51" s="4" t="n">
-        <v>15330.82</v>
+        <v>14906.23</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>15209.16</v>
+        <v>14994.58</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>-3292.04</v>
+        <v>-3506.63</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>-4070.19</v>
+        <v>-3900.77</v>
       </c>
       <c r="AD51" s="4" t="n">
-        <v>-3355.53</v>
+        <v>-3570.12</v>
       </c>
       <c r="AE51" s="4" t="n">
-        <v>-3622.03</v>
+        <v>-3836.62</v>
       </c>
       <c r="AF51" s="4" t="n">
-        <v>8287.969999999999</v>
+        <v>8073.39</v>
       </c>
       <c r="AG51" s="4" t="n">
-        <v>-2992.69</v>
+        <v>-3207.28</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-2891.89</v>
+        <v>-3490.47</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>-3457.74</v>
+        <v>-3710.33</v>
       </c>
       <c r="AJ51" s="4" t="n">
-        <v>-2796.6</v>
+        <v>-3011.18</v>
       </c>
       <c r="AK51" s="4" t="n">
-        <v>-3436.09</v>
+        <v>-3650.67</v>
       </c>
       <c r="AL51" s="4" t="n">
-        <v>5479.92</v>
+        <v>5679.92</v>
       </c>
       <c r="AM51" s="4" t="n">
         <v>10445.6</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>8913.15</v>
+        <v>6090.13</v>
       </c>
     </row>
     <row r="52">
@@ -6582,121 +6582,121 @@
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>2406.73</v>
+        <v>2571.73</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>4723.02</v>
+        <v>2293.02</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>12381.79</v>
+        <v>2056.79</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>11146.21</v>
+        <v>1835.21</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>10277.94</v>
+        <v>1271.94</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>9953.82</v>
+        <v>1037.82</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>9663.549999999999</v>
+        <v>822.55</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>9426.91</v>
+        <v>10640.91</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>9204.959999999999</v>
+        <v>9944.959999999999</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>8997.809999999999</v>
+        <v>9632.809999999999</v>
       </c>
       <c r="L52" s="4" t="n">
-        <v>8839.49</v>
+        <v>9294.49</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>8479.92</v>
+        <v>8679.92</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>7138.92</v>
+        <v>7338.92</v>
       </c>
       <c r="O52" s="4" t="n">
-        <v>25745.31</v>
+        <v>25945.31</v>
       </c>
       <c r="P52" s="4" t="n">
-        <v>25144.84</v>
+        <v>25344.84</v>
       </c>
       <c r="Q52" s="4" t="n">
-        <v>22868.72</v>
+        <v>23452.72</v>
       </c>
       <c r="R52" s="4" t="n">
-        <v>22199.72</v>
+        <v>22783.72</v>
       </c>
       <c r="S52" s="4" t="n">
-        <v>21689.56</v>
+        <v>22273.56</v>
       </c>
       <c r="T52" s="4" t="n">
-        <v>21250.79</v>
+        <v>21834.79</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>20880</v>
+        <v>21464</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>20591.77</v>
+        <v>20791.77</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>20337.58</v>
+        <v>20537.58</v>
       </c>
       <c r="X52" s="4" t="n">
-        <v>20077.94</v>
+        <v>20277.94</v>
       </c>
       <c r="Y52" s="4" t="n">
-        <v>18925.53</v>
+        <v>19125.53</v>
       </c>
       <c r="Z52" s="4" t="n">
-        <v>34256.35</v>
+        <v>34031.77</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>49465.51</v>
+        <v>49026.35</v>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>46173.47</v>
+        <v>45519.72</v>
       </c>
       <c r="AC52" s="4" t="n">
-        <v>42103.28</v>
+        <v>41618.95</v>
       </c>
       <c r="AD52" s="4" t="n">
-        <v>38747.75</v>
+        <v>38048.84</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>35125.72</v>
+        <v>34212.22</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>43413.69</v>
+        <v>42285.61</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>40421</v>
+        <v>39078.33</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>37529.1</v>
+        <v>35587.85</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>34071.36</v>
+        <v>31877.53</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>31274.76</v>
+        <v>28866.35</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>27838.68</v>
+        <v>25215.68</v>
       </c>
       <c r="AL52" s="4" t="n">
-        <v>8479.92</v>
+        <v>8679.92</v>
       </c>
       <c r="AM52" s="4" t="n">
-        <v>18925.53</v>
+        <v>19125.53</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>27838.68</v>
+        <v>25215.68</v>
       </c>
     </row>
     <row r="53">
@@ -6752,76 +6752,76 @@
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z54" s="4" t="n">
         <v>3</v>
@@ -6860,10 +6860,10 @@
         <v>3</v>
       </c>
       <c r="AL54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN54" s="4" t="n">
         <v>3</v>
@@ -6876,121 +6876,121 @@
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AB55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AC55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AD55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AE55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AF55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AG55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AH55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AI55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AJ55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AK55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
       <c r="AL55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN55" s="4" t="n">
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
     </row>
   </sheetData>
@@ -7055,13 +7055,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>83.33</v>
       </c>
       <c r="C3" t="n">
-        <v>575</v>
+        <v>508.33</v>
       </c>
       <c r="D3" t="n">
-        <v>1441.67</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="4">
@@ -7071,13 +7071,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>450</v>
+        <v>516.67</v>
       </c>
       <c r="C4" t="n">
-        <v>925</v>
+        <v>991.67</v>
       </c>
       <c r="D4" t="n">
-        <v>1258.33</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="5">
@@ -7119,13 +7119,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8479.92</v>
+        <v>8679.92</v>
       </c>
       <c r="C7" t="n">
-        <v>18925.53</v>
+        <v>19125.53</v>
       </c>
       <c r="D7" t="n">
-        <v>27838.68</v>
+        <v>25215.68</v>
       </c>
     </row>
     <row r="8">
@@ -7135,13 +7135,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8929.92</v>
+        <v>9196.59</v>
       </c>
       <c r="C8" t="n">
-        <v>39850.53</v>
+        <v>40117.2</v>
       </c>
       <c r="D8" t="n">
-        <v>49097.01</v>
+        <v>46540.68</v>
       </c>
     </row>
     <row r="9">
@@ -7170,10 +7170,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>619</v>
+        <v>657</v>
       </c>
       <c r="D10" t="n">
-        <v>671</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
@@ -7186,10 +7186,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>22285.67</v>
+        <v>22323.67</v>
       </c>
       <c r="D11" t="n">
-        <v>28337.67</v>
+        <v>27808.67</v>
       </c>
     </row>
     <row r="12">
@@ -7199,13 +7199,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8929.92</v>
+        <v>9196.59</v>
       </c>
       <c r="C12" t="n">
-        <v>17564.87</v>
+        <v>17793.53</v>
       </c>
       <c r="D12" t="n">
-        <v>20759.34</v>
+        <v>18732.01</v>
       </c>
     </row>
     <row r="13">
@@ -7231,13 +7231,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-5070.08</v>
+        <v>-4803.41</v>
       </c>
       <c r="C14" t="n">
-        <v>3564.87</v>
+        <v>3793.53</v>
       </c>
       <c r="D14" t="n">
-        <v>6759.34</v>
+        <v>4732.01</v>
       </c>
     </row>
     <row r="15">
@@ -7247,13 +7247,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8929.92</v>
+        <v>9196.59</v>
       </c>
       <c r="C15" t="n">
-        <v>17564.87</v>
+        <v>17793.53</v>
       </c>
       <c r="D15" t="n">
-        <v>20759.34</v>
+        <v>18732.01</v>
       </c>
     </row>
   </sheetData>
@@ -9662,7 +9662,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>0</v>
@@ -9758,7 +9758,7 @@
         <v>0</v>
       </c>
       <c r="AL22" s="4" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="AM22" s="4" t="n">
         <v>1200</v>
@@ -9910,7 +9910,7 @@
         <v>71.55</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>573.23</v>
+        <v>373.23</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>74.08</v>
@@ -10006,7 +10006,7 @@
         <v>952.5700000000001</v>
       </c>
       <c r="AL24" s="4" t="n">
-        <v>1389.57</v>
+        <v>1189.57</v>
       </c>
       <c r="AM24" s="4" t="n">
         <v>4053.07</v>
@@ -10034,7 +10034,7 @@
         <v>-56.58</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>-553.27</v>
+        <v>-353.27</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>-54.12</v>
@@ -10130,7 +10130,7 @@
         <v>13771.33</v>
       </c>
       <c r="AL25" s="4" t="n">
-        <v>-820.08</v>
+        <v>-620.08</v>
       </c>
       <c r="AM25" s="4" t="n">
         <v>32710.23</v>
@@ -10264,40 +10264,40 @@
         <v>0</v>
       </c>
       <c r="Z27" s="4" t="n">
-        <v>6083.33</v>
+        <v>7250</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AB27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AC27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AD27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AE27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AF27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AG27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AH27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AI27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AJ27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AK27" s="4" t="n">
-        <v>10250</v>
+        <v>11416.67</v>
       </c>
       <c r="AL27" s="4" t="n">
         <v>0</v>
@@ -10306,7 +10306,7 @@
         <v>0</v>
       </c>
       <c r="AN27" s="4" t="n">
-        <v>118833.33</v>
+        <v>132833.37</v>
       </c>
     </row>
     <row r="28">
@@ -10388,40 +10388,40 @@
         <v>0</v>
       </c>
       <c r="Z28" s="4" t="n">
-        <v>145.31</v>
+        <v>271.99</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AB28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AC28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AD28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AE28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AF28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AG28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AH28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AI28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AJ28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AK28" s="4" t="n">
-        <v>254.97</v>
+        <v>434.36</v>
       </c>
       <c r="AL28" s="4" t="n">
         <v>0</v>
@@ -10430,7 +10430,7 @@
         <v>0</v>
       </c>
       <c r="AN28" s="4" t="n">
-        <v>2949.98</v>
+        <v>5049.95</v>
       </c>
     </row>
     <row r="29">
@@ -10512,40 +10512,40 @@
         <v>0</v>
       </c>
       <c r="Z29" s="4" t="n">
-        <v>182.5</v>
+        <v>217.5</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AB29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AC29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AD29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AE29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AF29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AG29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AH29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AI29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AJ29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AK29" s="4" t="n">
-        <v>307.5</v>
+        <v>342.5</v>
       </c>
       <c r="AL29" s="4" t="n">
         <v>0</v>
@@ -10554,7 +10554,7 @@
         <v>0</v>
       </c>
       <c r="AN29" s="4" t="n">
-        <v>3565</v>
+        <v>3985</v>
       </c>
     </row>
     <row r="30">
@@ -10636,7 +10636,7 @@
         <v>0</v>
       </c>
       <c r="Z30" s="4" t="n">
-        <v>420</v>
+        <v>630</v>
       </c>
       <c r="AA30" s="4" t="n">
         <v>420</v>
@@ -10678,7 +10678,7 @@
         <v>0</v>
       </c>
       <c r="AN30" s="4" t="n">
-        <v>840</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="31">
@@ -10760,40 +10760,40 @@
         <v>0</v>
       </c>
       <c r="Z31" s="4" t="n">
-        <v>6831.14</v>
+        <v>8369.49</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>11232.47</v>
+        <v>12613.53</v>
       </c>
       <c r="AB31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AC31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AD31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AE31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AF31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AG31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AH31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AI31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AJ31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AK31" s="4" t="n">
-        <v>10812.47</v>
+        <v>12193.53</v>
       </c>
       <c r="AL31" s="4" t="n">
         <v>0</v>
@@ -10802,7 +10802,7 @@
         <v>0</v>
       </c>
       <c r="AN31" s="4" t="n">
-        <v>126188.31</v>
+        <v>142918.32</v>
       </c>
     </row>
     <row r="32">
@@ -10812,40 +10812,40 @@
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>240</v>
+        <v>75</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>210</v>
+        <v>75</v>
       </c>
       <c r="D32" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I32" s="4" t="n">
         <v>150</v>
       </c>
-      <c r="E32" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="F32" s="4" t="n">
-        <v>180</v>
-      </c>
-      <c r="G32" s="4" t="n">
-        <v>135</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="I32" s="4" t="n">
-        <v>75</v>
-      </c>
       <c r="J32" s="4" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>45</v>
+        <v>150</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>45</v>
+        <v>225</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>195</v>
+        <v>450</v>
       </c>
       <c r="N32" s="4" t="n">
         <v>840</v>
@@ -11559,28 +11559,28 @@
         <v>52</v>
       </c>
       <c r="C38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="4" t="n">
         <v>270</v>
       </c>
-      <c r="D38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="4" t="n">
+      <c r="J38" s="4" t="n">
         <v>384</v>
-      </c>
-      <c r="F38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="K38" s="4" t="n">
         <v>0</v>
@@ -11601,22 +11601,22 @@
         <v>0</v>
       </c>
       <c r="Q38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" s="4" t="n">
         <v>384</v>
-      </c>
-      <c r="R38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V38" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="W38" s="4" t="n">
         <v>0</v>
@@ -11637,22 +11637,22 @@
         <v>0</v>
       </c>
       <c r="AC38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH38" s="4" t="n">
         <v>384</v>
-      </c>
-      <c r="AD38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH38" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="AI38" s="4" t="n">
         <v>0</v>
@@ -11928,40 +11928,40 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>-593.27</v>
+        <v>-428.27</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>-683.71</v>
+        <v>-278.71</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>-341.23</v>
+        <v>-236.23</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>-635.58</v>
+        <v>-221.58</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>-868.27</v>
+        <v>-563.27</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-324.12</v>
+        <v>-234.12</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>-290.27</v>
+        <v>-215.27</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>-236.64</v>
+        <v>-581.64</v>
       </c>
       <c r="J41" s="4" t="n">
-        <v>-221.95</v>
+        <v>-695.95</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>-207.15</v>
+        <v>-312.15</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>-158.32</v>
+        <v>-338.32</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>-359.57</v>
+        <v>-614.5700000000001</v>
       </c>
       <c r="N41" s="4" t="n">
         <v>-1622.11</v>
@@ -11973,7 +11973,7 @@
         <v>944.47</v>
       </c>
       <c r="Q41" s="4" t="n">
-        <v>277.13</v>
+        <v>661.13</v>
       </c>
       <c r="R41" s="4" t="n">
         <v>1904.98</v>
@@ -11988,7 +11988,7 @@
         <v>2923.81</v>
       </c>
       <c r="V41" s="4" t="n">
-        <v>3022.82</v>
+        <v>2638.82</v>
       </c>
       <c r="W41" s="4" t="n">
         <v>3069.19</v>
@@ -12000,49 +12000,49 @@
         <v>2000.07</v>
       </c>
       <c r="Z41" s="4" t="n">
-        <v>-3918.96</v>
+        <v>-5457.31</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>-6001.77</v>
+        <v>-7382.83</v>
       </c>
       <c r="AB41" s="4" t="n">
-        <v>-4441.28</v>
+        <v>-5822.34</v>
       </c>
       <c r="AC41" s="4" t="n">
-        <v>-2971.43</v>
+        <v>-3968.49</v>
       </c>
       <c r="AD41" s="4" t="n">
-        <v>-2138.32</v>
+        <v>-3519.38</v>
       </c>
       <c r="AE41" s="4" t="n">
-        <v>-2225.33</v>
+        <v>-3606.39</v>
       </c>
       <c r="AF41" s="4" t="n">
-        <v>-170</v>
+        <v>-1551.06</v>
       </c>
       <c r="AG41" s="4" t="n">
-        <v>1262.61</v>
+        <v>-118.45</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>1418.46</v>
+        <v>-346.6</v>
       </c>
       <c r="AI41" s="4" t="n">
-        <v>1528.41</v>
+        <v>147.35</v>
       </c>
       <c r="AJ41" s="4" t="n">
-        <v>1562.83</v>
+        <v>181.77</v>
       </c>
       <c r="AK41" s="4" t="n">
-        <v>325.03</v>
+        <v>-1056.03</v>
       </c>
       <c r="AL41" s="4" t="n">
-        <v>-4920.08</v>
+        <v>-4720.08</v>
       </c>
       <c r="AM41" s="4" t="n">
         <v>21199.24</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-15769.75</v>
+        <v>-32499.76</v>
       </c>
     </row>
     <row r="42">
@@ -12061,16 +12061,16 @@
         <v>0</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="H42" s="4" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="I42" s="4" t="n">
         <v>16.67</v>
@@ -12160,7 +12160,7 @@
         <v>145.83</v>
       </c>
       <c r="AL42" s="4" t="n">
-        <v>150.03</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="AM42" s="4" t="n">
         <v>425.04</v>
@@ -12176,40 +12176,40 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>-593.27</v>
+        <v>-428.27</v>
       </c>
       <c r="C43" s="4" t="n">
-        <v>-683.71</v>
+        <v>-278.71</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>-341.23</v>
+        <v>-236.23</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>-652.24</v>
+        <v>-221.58</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>-884.9400000000001</v>
+        <v>-563.27</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>-340.79</v>
+        <v>-234.12</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>-306.93</v>
+        <v>-215.27</v>
       </c>
       <c r="I43" s="4" t="n">
-        <v>-253.31</v>
+        <v>-598.3099999999999</v>
       </c>
       <c r="J43" s="4" t="n">
-        <v>-238.62</v>
+        <v>-712.62</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>-223.82</v>
+        <v>-328.82</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>-174.98</v>
+        <v>-354.98</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>-376.24</v>
+        <v>-631.24</v>
       </c>
       <c r="N43" s="4" t="n">
         <v>-1638.77</v>
@@ -12221,7 +12221,7 @@
         <v>927.8099999999999</v>
       </c>
       <c r="Q43" s="4" t="n">
-        <v>235.46</v>
+        <v>619.46</v>
       </c>
       <c r="R43" s="4" t="n">
         <v>1863.32</v>
@@ -12236,7 +12236,7 @@
         <v>2882.14</v>
       </c>
       <c r="V43" s="4" t="n">
-        <v>2981.16</v>
+        <v>2597.16</v>
       </c>
       <c r="W43" s="4" t="n">
         <v>3027.52</v>
@@ -12248,49 +12248,49 @@
         <v>1958.4</v>
       </c>
       <c r="Z43" s="4" t="n">
-        <v>-4041.18</v>
+        <v>-5579.53</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>-6147.6</v>
+        <v>-7528.66</v>
       </c>
       <c r="AB43" s="4" t="n">
-        <v>-4587.11</v>
+        <v>-5968.17</v>
       </c>
       <c r="AC43" s="4" t="n">
-        <v>-3117.26</v>
+        <v>-4114.32</v>
       </c>
       <c r="AD43" s="4" t="n">
-        <v>-2284.15</v>
+        <v>-3665.21</v>
       </c>
       <c r="AE43" s="4" t="n">
-        <v>-2371.16</v>
+        <v>-3752.22</v>
       </c>
       <c r="AF43" s="4" t="n">
-        <v>-315.83</v>
+        <v>-1696.89</v>
       </c>
       <c r="AG43" s="4" t="n">
-        <v>1116.78</v>
+        <v>-264.28</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>1272.63</v>
+        <v>-492.43</v>
       </c>
       <c r="AI43" s="4" t="n">
-        <v>1382.57</v>
+        <v>1.51</v>
       </c>
       <c r="AJ43" s="4" t="n">
-        <v>1417</v>
+        <v>35.94</v>
       </c>
       <c r="AK43" s="4" t="n">
-        <v>179.19</v>
+        <v>-1201.86</v>
       </c>
       <c r="AL43" s="4" t="n">
-        <v>-5070.08</v>
+        <v>-4803.42</v>
       </c>
       <c r="AM43" s="4" t="n">
         <v>20774.25</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-17496.12</v>
+        <v>-34226.12</v>
       </c>
     </row>
     <row r="44">
@@ -12603,19 +12603,19 @@
         <v>0</v>
       </c>
       <c r="E47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4" t="n">
         <v>600</v>
-      </c>
-      <c r="F47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="J47" s="4" t="n">
         <v>0</v>
@@ -12817,7 +12817,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>2808</v>
+        <v>2846</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -12832,7 +12832,7 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>2808</v>
+        <v>2846</v>
       </c>
     </row>
     <row r="49">
@@ -12845,10 +12845,10 @@
         <v>0</v>
       </c>
       <c r="C49" s="4" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>0</v>
@@ -12863,7 +12863,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="4" t="n">
-        <v>0</v>
+        <v>11000</v>
       </c>
       <c r="J49" s="4" t="n">
         <v>0</v>
@@ -12966,40 +12966,40 @@
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>593.27</v>
+        <v>428.27</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>683.71</v>
+        <v>278.71</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>356.2</v>
+        <v>251.2</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>1250.55</v>
+        <v>236.55</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>888.23</v>
+        <v>583.23</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>344.08</v>
+        <v>254.08</v>
       </c>
       <c r="H50" s="4" t="n">
-        <v>315.22</v>
+        <v>240.22</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>311.58</v>
+        <v>1256.58</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>296.89</v>
+        <v>770.89</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>282.09</v>
+        <v>387.09</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>283.25</v>
+        <v>463.25</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>484.5</v>
+        <v>739.5</v>
       </c>
       <c r="N50" s="4" t="n">
         <v>1816.99</v>
@@ -13011,7 +13011,7 @@
         <v>1056.97</v>
       </c>
       <c r="Q50" s="4" t="n">
-        <v>2629.31</v>
+        <v>2245.31</v>
       </c>
       <c r="R50" s="4" t="n">
         <v>1838.07</v>
@@ -13026,7 +13026,7 @@
         <v>889.2</v>
       </c>
       <c r="V50" s="4" t="n">
-        <v>840.17</v>
+        <v>1224.17</v>
       </c>
       <c r="W50" s="4" t="n">
         <v>788.8200000000001</v>
@@ -13038,49 +13038,49 @@
         <v>1877.9</v>
       </c>
       <c r="Z50" s="4" t="n">
-        <v>14478.45</v>
+        <v>16016.8</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>15969.43</v>
+        <v>17350.49</v>
       </c>
       <c r="AB50" s="4" t="n">
-        <v>13653.84</v>
+        <v>15034.9</v>
       </c>
       <c r="AC50" s="4" t="n">
-        <v>14738.97</v>
+        <v>15736.03</v>
       </c>
       <c r="AD50" s="4" t="n">
-        <v>14005.75</v>
+        <v>15386.81</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>14072.71</v>
+        <v>15453.77</v>
       </c>
       <c r="AF50" s="4" t="n">
-        <v>14754</v>
+        <v>16135.06</v>
       </c>
       <c r="AG50" s="4" t="n">
-        <v>13326.38</v>
+        <v>14707.44</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>13215.53</v>
+        <v>14980.59</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>15908.59</v>
+        <v>17327.65</v>
       </c>
       <c r="AJ50" s="4" t="n">
-        <v>13106.18</v>
+        <v>14487.24</v>
       </c>
       <c r="AK50" s="4" t="n">
-        <v>14398.87</v>
+        <v>15779.93</v>
       </c>
       <c r="AL50" s="4" t="n">
-        <v>6089.57</v>
+        <v>5889.57</v>
       </c>
       <c r="AM50" s="4" t="n">
         <v>16464.08</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>171628.7</v>
+        <v>188396.71</v>
       </c>
     </row>
     <row r="51">
@@ -13090,40 +13090,40 @@
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>-593.27</v>
+        <v>-428.27</v>
       </c>
       <c r="C51" s="4" t="n">
-        <v>2316.29</v>
+        <v>-278.71</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>7658.77</v>
+        <v>-236.23</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>-1235.58</v>
+        <v>-221.58</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>-868.27</v>
+        <v>-563.27</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>-324.12</v>
+        <v>-234.12</v>
       </c>
       <c r="H51" s="4" t="n">
-        <v>-290.27</v>
+        <v>-215.27</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>-236.64</v>
+        <v>9818.360000000001</v>
       </c>
       <c r="J51" s="4" t="n">
-        <v>-221.95</v>
+        <v>-695.95</v>
       </c>
       <c r="K51" s="4" t="n">
-        <v>-207.15</v>
+        <v>-312.15</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>-158.32</v>
+        <v>-338.32</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>-359.57</v>
+        <v>-614.5700000000001</v>
       </c>
       <c r="N51" s="4" t="n">
         <v>-1622.11</v>
@@ -13135,7 +13135,7 @@
         <v>-722.1900000000001</v>
       </c>
       <c r="Q51" s="4" t="n">
-        <v>-2289.54</v>
+        <v>-1905.54</v>
       </c>
       <c r="R51" s="4" t="n">
         <v>18571.65</v>
@@ -13150,7 +13150,7 @@
         <v>-409.53</v>
       </c>
       <c r="V51" s="4" t="n">
-        <v>-310.51</v>
+        <v>-694.51</v>
       </c>
       <c r="W51" s="4" t="n">
         <v>-264.15</v>
@@ -13162,49 +13162,49 @@
         <v>-1333.27</v>
       </c>
       <c r="Z51" s="4" t="n">
-        <v>30181.04</v>
+        <v>28642.69</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>20814.9</v>
+        <v>19433.84</v>
       </c>
       <c r="AB51" s="4" t="n">
-        <v>-12774.61</v>
+        <v>-14155.67</v>
       </c>
       <c r="AC51" s="4" t="n">
-        <v>16195.24</v>
+        <v>15198.18</v>
       </c>
       <c r="AD51" s="4" t="n">
-        <v>7028.35</v>
+        <v>5647.29</v>
       </c>
       <c r="AE51" s="4" t="n">
-        <v>-13058.66</v>
+        <v>-14439.72</v>
       </c>
       <c r="AF51" s="4" t="n">
-        <v>18330</v>
+        <v>16948.94</v>
       </c>
       <c r="AG51" s="4" t="n">
-        <v>-12237.39</v>
+        <v>-13618.45</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-12081.54</v>
+        <v>-13846.6</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>-14779.59</v>
+        <v>-16198.65</v>
       </c>
       <c r="AJ51" s="4" t="n">
-        <v>-11937.17</v>
+        <v>-13318.23</v>
       </c>
       <c r="AK51" s="4" t="n">
-        <v>-13174.97</v>
+        <v>-14556.03</v>
       </c>
       <c r="AL51" s="4" t="n">
-        <v>5479.92</v>
+        <v>5679.92</v>
       </c>
       <c r="AM51" s="4" t="n">
         <v>28632.56</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>2505.6</v>
+        <v>-14262.41</v>
       </c>
     </row>
     <row r="52">
@@ -13214,121 +13214,121 @@
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>2406.73</v>
+        <v>2571.73</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>4723.02</v>
+        <v>2293.02</v>
       </c>
       <c r="D52" s="4" t="n">
-        <v>12381.79</v>
+        <v>2056.79</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>11146.21</v>
+        <v>1835.21</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>10277.94</v>
+        <v>1271.94</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>9953.82</v>
+        <v>1037.82</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>9663.549999999999</v>
+        <v>822.55</v>
       </c>
       <c r="I52" s="4" t="n">
-        <v>9426.91</v>
+        <v>10640.91</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>9204.959999999999</v>
+        <v>9944.959999999999</v>
       </c>
       <c r="K52" s="4" t="n">
-        <v>8997.809999999999</v>
+        <v>9632.809999999999</v>
       </c>
       <c r="L52" s="4" t="n">
-        <v>8839.49</v>
+        <v>9294.49</v>
       </c>
       <c r="M52" s="4" t="n">
-        <v>8479.92</v>
+        <v>8679.92</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>6857.82</v>
+        <v>7057.82</v>
       </c>
       <c r="O52" s="4" t="n">
-        <v>25271.31</v>
+        <v>25471.31</v>
       </c>
       <c r="P52" s="4" t="n">
-        <v>24549.12</v>
+        <v>24749.12</v>
       </c>
       <c r="Q52" s="4" t="n">
-        <v>22259.58</v>
+        <v>22843.58</v>
       </c>
       <c r="R52" s="4" t="n">
-        <v>40831.23</v>
+        <v>41415.23</v>
       </c>
       <c r="S52" s="4" t="n">
-        <v>40211.35</v>
+        <v>40795.35</v>
       </c>
       <c r="T52" s="4" t="n">
-        <v>39695.75</v>
+        <v>40279.75</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>39286.22</v>
+        <v>39870.22</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>38975.71</v>
+        <v>39175.71</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>38711.57</v>
+        <v>38911.57</v>
       </c>
       <c r="X52" s="4" t="n">
-        <v>38445.76</v>
+        <v>38645.76</v>
       </c>
       <c r="Y52" s="4" t="n">
-        <v>37112.49</v>
+        <v>37312.49</v>
       </c>
       <c r="Z52" s="4" t="n">
-        <v>67293.53</v>
+        <v>65955.17999999999</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>88108.42999999999</v>
+        <v>85389.03</v>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>75333.82000000001</v>
+        <v>71233.36</v>
       </c>
       <c r="AC52" s="4" t="n">
-        <v>91529.06</v>
+        <v>86431.53999999999</v>
       </c>
       <c r="AD52" s="4" t="n">
-        <v>98557.41</v>
+        <v>92078.83</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>85498.75</v>
+        <v>77639.11</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>103828.75</v>
+        <v>94588.05</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>91591.36</v>
+        <v>80969.60000000001</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>79509.82000000001</v>
+        <v>67123</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>64730.23</v>
+        <v>50924.35</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>52793.06</v>
+        <v>37606.12</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>39618.09</v>
+        <v>23050.09</v>
       </c>
       <c r="AL52" s="4" t="n">
-        <v>8479.92</v>
+        <v>8679.92</v>
       </c>
       <c r="AM52" s="4" t="n">
-        <v>37112.49</v>
+        <v>37312.49</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>39618.09</v>
+        <v>23050.09</v>
       </c>
     </row>
     <row r="53">
@@ -13384,76 +13384,76 @@
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z54" s="4" t="n">
         <v>4</v>
@@ -13492,10 +13492,10 @@
         <v>6</v>
       </c>
       <c r="AL54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN54" s="4" t="n">
         <v>6</v>
@@ -13508,76 +13508,76 @@
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z55" s="4" t="n">
         <v>3.25</v>
@@ -13616,10 +13616,10 @@
         <v>5.25</v>
       </c>
       <c r="AL55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN55" s="4" t="n">
         <v>5.25</v>
@@ -13687,13 +13687,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>83.33</v>
       </c>
       <c r="C3" t="n">
-        <v>575</v>
+        <v>508.33</v>
       </c>
       <c r="D3" t="n">
-        <v>2301.39</v>
+        <v>2234.72</v>
       </c>
     </row>
     <row r="4">
@@ -13703,13 +13703,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>450</v>
+        <v>516.67</v>
       </c>
       <c r="C4" t="n">
-        <v>925</v>
+        <v>991.67</v>
       </c>
       <c r="D4" t="n">
-        <v>2948.61</v>
+        <v>3015.28</v>
       </c>
     </row>
     <row r="5">
@@ -13751,13 +13751,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8479.92</v>
+        <v>8679.92</v>
       </c>
       <c r="C7" t="n">
-        <v>37112.49</v>
+        <v>37312.49</v>
       </c>
       <c r="D7" t="n">
-        <v>39618.09</v>
+        <v>23050.09</v>
       </c>
     </row>
     <row r="8">
@@ -13767,13 +13767,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8929.92</v>
+        <v>9196.59</v>
       </c>
       <c r="C8" t="n">
-        <v>82037.49000000001</v>
+        <v>82304.16</v>
       </c>
       <c r="D8" t="n">
-        <v>86566.7</v>
+        <v>70065.36</v>
       </c>
     </row>
     <row r="9">
@@ -13802,7 +13802,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>2808</v>
+        <v>2846</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -13818,7 +13818,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>55141.33</v>
+        <v>55179.33</v>
       </c>
       <c r="D11" t="n">
         <v>77166.67</v>
@@ -13831,13 +13831,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8929.92</v>
+        <v>9196.59</v>
       </c>
       <c r="C12" t="n">
-        <v>26896.16</v>
+        <v>27124.82</v>
       </c>
       <c r="D12" t="n">
-        <v>9400.030000000001</v>
+        <v>-7101.3</v>
       </c>
     </row>
     <row r="13">
@@ -13863,13 +13863,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-5070.08</v>
+        <v>-4803.41</v>
       </c>
       <c r="C14" t="n">
-        <v>12896.16</v>
+        <v>13124.82</v>
       </c>
       <c r="D14" t="n">
-        <v>-4599.97</v>
+        <v>-21101.3</v>
       </c>
     </row>
     <row r="15">
@@ -13879,13 +13879,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8929.92</v>
+        <v>9196.59</v>
       </c>
       <c r="C15" t="n">
-        <v>26896.16</v>
+        <v>27124.82</v>
       </c>
       <c r="D15" t="n">
-        <v>9400.030000000001</v>
+        <v>-7101.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business plan v6: add barriers to entry and IP section
New section 3.4 covering protected algorithms (trade secrets), proprietary
dataset, exclusive partnerships and patents/trademarks, with status vs plan.
Patent search (Y2) and UK filing (Y3) costs added to the model.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146q3FtAYmgQ1rtNsNNpdiD
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
@@ -4733,7 +4733,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="V36" s="4" t="n">
         <v>0</v>
@@ -4763,7 +4763,7 @@
         <v>0</v>
       </c>
       <c r="AE36" s="4" t="n">
-        <v>400</v>
+        <v>1900</v>
       </c>
       <c r="AF36" s="4" t="n">
         <v>0</v>
@@ -4787,10 +4787,10 @@
         <v>0</v>
       </c>
       <c r="AM36" s="4" t="n">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>400</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="37">
@@ -5353,7 +5353,7 @@
         <v>1227.9</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>1295.88</v>
+        <v>695.88</v>
       </c>
       <c r="V41" s="4" t="n">
         <v>994.4400000000001</v>
@@ -5383,7 +5383,7 @@
         <v>-236.78</v>
       </c>
       <c r="AE41" s="4" t="n">
-        <v>-503.28</v>
+        <v>-2003.28</v>
       </c>
       <c r="AF41" s="4" t="n">
         <v>406.72</v>
@@ -5407,10 +5407,10 @@
         <v>-4720.08</v>
       </c>
       <c r="AM41" s="4" t="n">
-        <v>9678.940000000001</v>
+        <v>9078.940000000001</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>1947.15</v>
+        <v>447.15</v>
       </c>
     </row>
     <row r="42">
@@ -5601,7 +5601,7 @@
         <v>1186.23</v>
       </c>
       <c r="U43" s="4" t="n">
-        <v>1254.21</v>
+        <v>654.21</v>
       </c>
       <c r="V43" s="4" t="n">
         <v>952.77</v>
@@ -5631,7 +5631,7 @@
         <v>-311.78</v>
       </c>
       <c r="AE43" s="4" t="n">
-        <v>-578.28</v>
+        <v>-2078.28</v>
       </c>
       <c r="AF43" s="4" t="n">
         <v>331.72</v>
@@ -5655,10 +5655,10 @@
         <v>-4803.42</v>
       </c>
       <c r="AM43" s="4" t="n">
-        <v>9253.940000000001</v>
+        <v>8653.940000000001</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>1080.48</v>
+        <v>-419.52</v>
       </c>
     </row>
     <row r="44">
@@ -6185,7 +6185,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>657</v>
+        <v>543</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -6200,7 +6200,7 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>657</v>
+        <v>543</v>
       </c>
     </row>
     <row r="49">
@@ -6391,7 +6391,7 @@
         <v>778.54</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>710.5599999999999</v>
+        <v>1310.56</v>
       </c>
       <c r="V50" s="4" t="n">
         <v>1061.99</v>
@@ -6421,7 +6421,7 @@
         <v>4269.53</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>4501.01</v>
+        <v>6001.01</v>
       </c>
       <c r="AF50" s="4" t="n">
         <v>4650.97</v>
@@ -6433,7 +6433,7 @@
         <v>4264.82</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>4479.69</v>
+        <v>4365.69</v>
       </c>
       <c r="AJ50" s="4" t="n">
         <v>3825.54</v>
@@ -6445,10 +6445,10 @@
         <v>5889.57</v>
       </c>
       <c r="AM50" s="4" t="n">
-        <v>13331.97</v>
+        <v>13931.97</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>54217.87</v>
+        <v>55603.87</v>
       </c>
     </row>
     <row r="51">
@@ -6515,7 +6515,7 @@
         <v>-438.77</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>-370.79</v>
+        <v>-970.79</v>
       </c>
       <c r="V51" s="4" t="n">
         <v>-672.23</v>
@@ -6545,7 +6545,7 @@
         <v>-3570.12</v>
       </c>
       <c r="AE51" s="4" t="n">
-        <v>-3836.62</v>
+        <v>-5336.62</v>
       </c>
       <c r="AF51" s="4" t="n">
         <v>8073.39</v>
@@ -6557,7 +6557,7 @@
         <v>-3490.47</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>-3710.33</v>
+        <v>-3596.33</v>
       </c>
       <c r="AJ51" s="4" t="n">
         <v>-3011.18</v>
@@ -6569,10 +6569,10 @@
         <v>5679.92</v>
       </c>
       <c r="AM51" s="4" t="n">
-        <v>10445.6</v>
+        <v>9845.6</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>6090.13</v>
+        <v>4704.13</v>
       </c>
     </row>
     <row r="52">
@@ -6639,64 +6639,64 @@
         <v>21834.79</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>21464</v>
+        <v>20864</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>20791.77</v>
+        <v>20191.77</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>20537.58</v>
+        <v>19937.58</v>
       </c>
       <c r="X52" s="4" t="n">
-        <v>20277.94</v>
+        <v>19677.94</v>
       </c>
       <c r="Y52" s="4" t="n">
-        <v>19125.53</v>
+        <v>18525.53</v>
       </c>
       <c r="Z52" s="4" t="n">
-        <v>34031.77</v>
+        <v>33431.77</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>49026.35</v>
+        <v>48426.35</v>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>45519.72</v>
+        <v>44919.72</v>
       </c>
       <c r="AC52" s="4" t="n">
-        <v>41618.95</v>
+        <v>41018.95</v>
       </c>
       <c r="AD52" s="4" t="n">
-        <v>38048.84</v>
+        <v>37448.84</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>34212.22</v>
+        <v>32112.22</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>42285.61</v>
+        <v>40185.61</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>39078.33</v>
+        <v>36978.33</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>35587.85</v>
+        <v>33487.85</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>31877.53</v>
+        <v>29891.53</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>28866.35</v>
+        <v>26880.35</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>25215.68</v>
+        <v>23229.68</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
       </c>
       <c r="AM52" s="4" t="n">
-        <v>19125.53</v>
+        <v>18525.53</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>25215.68</v>
+        <v>23229.68</v>
       </c>
     </row>
     <row r="53">
@@ -7122,10 +7122,10 @@
         <v>8679.92</v>
       </c>
       <c r="C7" t="n">
-        <v>19125.53</v>
+        <v>18525.53</v>
       </c>
       <c r="D7" t="n">
-        <v>25215.68</v>
+        <v>23229.68</v>
       </c>
     </row>
     <row r="8">
@@ -7138,10 +7138,10 @@
         <v>9196.59</v>
       </c>
       <c r="C8" t="n">
-        <v>40117.2</v>
+        <v>39517.2</v>
       </c>
       <c r="D8" t="n">
-        <v>46540.68</v>
+        <v>44554.68</v>
       </c>
     </row>
     <row r="9">
@@ -7170,10 +7170,10 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>657</v>
+        <v>543</v>
       </c>
       <c r="D10" t="n">
-        <v>142</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -7186,10 +7186,10 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>22323.67</v>
+        <v>22209.67</v>
       </c>
       <c r="D11" t="n">
-        <v>27808.67</v>
+        <v>27666.67</v>
       </c>
     </row>
     <row r="12">
@@ -7202,10 +7202,10 @@
         <v>9196.59</v>
       </c>
       <c r="C12" t="n">
-        <v>17793.53</v>
+        <v>17307.53</v>
       </c>
       <c r="D12" t="n">
-        <v>18732.01</v>
+        <v>16888.01</v>
       </c>
     </row>
     <row r="13">
@@ -7234,10 +7234,10 @@
         <v>-4803.41</v>
       </c>
       <c r="C14" t="n">
-        <v>3793.53</v>
+        <v>3307.53</v>
       </c>
       <c r="D14" t="n">
-        <v>4732.01</v>
+        <v>2888.01</v>
       </c>
     </row>
     <row r="15">
@@ -7250,10 +7250,10 @@
         <v>9196.59</v>
       </c>
       <c r="C15" t="n">
-        <v>17793.53</v>
+        <v>17307.53</v>
       </c>
       <c r="D15" t="n">
-        <v>18732.01</v>
+        <v>16888.01</v>
       </c>
     </row>
   </sheetData>
@@ -11365,7 +11365,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="V36" s="4" t="n">
         <v>0</v>
@@ -11395,7 +11395,7 @@
         <v>0</v>
       </c>
       <c r="AE36" s="4" t="n">
-        <v>400</v>
+        <v>1900</v>
       </c>
       <c r="AF36" s="4" t="n">
         <v>0</v>
@@ -11419,10 +11419,10 @@
         <v>0</v>
       </c>
       <c r="AM36" s="4" t="n">
-        <v>900</v>
+        <v>1500</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>400</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="37">
@@ -11985,7 +11985,7 @@
         <v>2817.73</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>2923.81</v>
+        <v>2323.81</v>
       </c>
       <c r="V41" s="4" t="n">
         <v>2638.82</v>
@@ -12015,7 +12015,7 @@
         <v>-3519.38</v>
       </c>
       <c r="AE41" s="4" t="n">
-        <v>-3606.39</v>
+        <v>-5106.39</v>
       </c>
       <c r="AF41" s="4" t="n">
         <v>-1551.06</v>
@@ -12039,10 +12039,10 @@
         <v>-4720.08</v>
       </c>
       <c r="AM41" s="4" t="n">
-        <v>21199.24</v>
+        <v>20599.24</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-32499.76</v>
+        <v>-33999.76</v>
       </c>
     </row>
     <row r="42">
@@ -12233,7 +12233,7 @@
         <v>2776.06</v>
       </c>
       <c r="U43" s="4" t="n">
-        <v>2882.14</v>
+        <v>2282.14</v>
       </c>
       <c r="V43" s="4" t="n">
         <v>2597.16</v>
@@ -12263,7 +12263,7 @@
         <v>-3665.21</v>
       </c>
       <c r="AE43" s="4" t="n">
-        <v>-3752.22</v>
+        <v>-5252.22</v>
       </c>
       <c r="AF43" s="4" t="n">
         <v>-1696.89</v>
@@ -12287,10 +12287,10 @@
         <v>-4803.42</v>
       </c>
       <c r="AM43" s="4" t="n">
-        <v>20774.25</v>
+        <v>20174.25</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-34226.12</v>
+        <v>-35726.12</v>
       </c>
     </row>
     <row r="44">
@@ -12817,7 +12817,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>2846</v>
+        <v>2732</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -12832,7 +12832,7 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>2846</v>
+        <v>2732</v>
       </c>
     </row>
     <row r="49">
@@ -13023,7 +13023,7 @@
         <v>990.28</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>889.2</v>
+        <v>1489.2</v>
       </c>
       <c r="V50" s="4" t="n">
         <v>1224.17</v>
@@ -13053,7 +13053,7 @@
         <v>15386.81</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>15453.77</v>
+        <v>16953.77</v>
       </c>
       <c r="AF50" s="4" t="n">
         <v>16135.06</v>
@@ -13065,7 +13065,7 @@
         <v>14980.59</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>17327.65</v>
+        <v>17213.65</v>
       </c>
       <c r="AJ50" s="4" t="n">
         <v>14487.24</v>
@@ -13077,10 +13077,10 @@
         <v>5889.57</v>
       </c>
       <c r="AM50" s="4" t="n">
-        <v>16464.08</v>
+        <v>17064.08</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>188396.71</v>
+        <v>189782.71</v>
       </c>
     </row>
     <row r="51">
@@ -13147,7 +13147,7 @@
         <v>-515.6</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>-409.53</v>
+        <v>-1009.53</v>
       </c>
       <c r="V51" s="4" t="n">
         <v>-694.51</v>
@@ -13177,7 +13177,7 @@
         <v>5647.29</v>
       </c>
       <c r="AE51" s="4" t="n">
-        <v>-14439.72</v>
+        <v>-15939.72</v>
       </c>
       <c r="AF51" s="4" t="n">
         <v>16948.94</v>
@@ -13189,7 +13189,7 @@
         <v>-13846.6</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>-16198.65</v>
+        <v>-16084.65</v>
       </c>
       <c r="AJ51" s="4" t="n">
         <v>-13318.23</v>
@@ -13201,10 +13201,10 @@
         <v>5679.92</v>
       </c>
       <c r="AM51" s="4" t="n">
-        <v>28632.56</v>
+        <v>28032.56</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>-14262.41</v>
+        <v>-15648.41</v>
       </c>
     </row>
     <row r="52">
@@ -13271,64 +13271,64 @@
         <v>40279.75</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>39870.22</v>
+        <v>39270.22</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>39175.71</v>
+        <v>38575.71</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>38911.57</v>
+        <v>38311.57</v>
       </c>
       <c r="X52" s="4" t="n">
-        <v>38645.76</v>
+        <v>38045.76</v>
       </c>
       <c r="Y52" s="4" t="n">
-        <v>37312.49</v>
+        <v>36712.49</v>
       </c>
       <c r="Z52" s="4" t="n">
-        <v>65955.17999999999</v>
+        <v>65355.18</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>85389.03</v>
+        <v>84789.03</v>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>71233.36</v>
+        <v>70633.36</v>
       </c>
       <c r="AC52" s="4" t="n">
-        <v>86431.53999999999</v>
+        <v>85831.53999999999</v>
       </c>
       <c r="AD52" s="4" t="n">
-        <v>92078.83</v>
+        <v>91478.83</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>77639.11</v>
+        <v>75539.11</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>94588.05</v>
+        <v>92488.05</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>80969.60000000001</v>
+        <v>78869.60000000001</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>67123</v>
+        <v>65023</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>50924.35</v>
+        <v>48938.35</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>37606.12</v>
+        <v>35620.12</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>23050.09</v>
+        <v>21064.09</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
       </c>
       <c r="AM52" s="4" t="n">
-        <v>37312.49</v>
+        <v>36712.49</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>23050.09</v>
+        <v>21064.09</v>
       </c>
     </row>
     <row r="53">
@@ -13754,10 +13754,10 @@
         <v>8679.92</v>
       </c>
       <c r="C7" t="n">
-        <v>37312.49</v>
+        <v>36712.49</v>
       </c>
       <c r="D7" t="n">
-        <v>23050.09</v>
+        <v>21064.09</v>
       </c>
     </row>
     <row r="8">
@@ -13770,10 +13770,10 @@
         <v>9196.59</v>
       </c>
       <c r="C8" t="n">
-        <v>82304.16</v>
+        <v>81704.16</v>
       </c>
       <c r="D8" t="n">
-        <v>70065.36</v>
+        <v>68079.36</v>
       </c>
     </row>
     <row r="9">
@@ -13802,7 +13802,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>2846</v>
+        <v>2732</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -13818,7 +13818,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>55179.33</v>
+        <v>55065.33</v>
       </c>
       <c r="D11" t="n">
         <v>77166.67</v>
@@ -13834,10 +13834,10 @@
         <v>9196.59</v>
       </c>
       <c r="C12" t="n">
-        <v>27124.82</v>
+        <v>26638.82</v>
       </c>
       <c r="D12" t="n">
-        <v>-7101.3</v>
+        <v>-9087.299999999999</v>
       </c>
     </row>
     <row r="13">
@@ -13866,10 +13866,10 @@
         <v>-4803.41</v>
       </c>
       <c r="C14" t="n">
-        <v>13124.82</v>
+        <v>12638.82</v>
       </c>
       <c r="D14" t="n">
-        <v>-21101.3</v>
+        <v>-23087.3</v>
       </c>
     </row>
     <row r="15">
@@ -13882,10 +13882,10 @@
         <v>9196.59</v>
       </c>
       <c r="C15" t="n">
-        <v>27124.82</v>
+        <v>26638.82</v>
       </c>
       <c r="D15" t="n">
-        <v>-7101.3</v>
+        <v>-9087.299999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business plan v6: patent attorney consulted; patent exploration in Year 3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146q3FtAYmgQ1rtNsNNpdiD
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
@@ -4733,7 +4733,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="V36" s="4" t="n">
         <v>0</v>
@@ -4751,7 +4751,7 @@
         <v>0</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="AB36" s="4" t="n">
         <v>0</v>
@@ -4763,7 +4763,7 @@
         <v>0</v>
       </c>
       <c r="AE36" s="4" t="n">
-        <v>1900</v>
+        <v>400</v>
       </c>
       <c r="AF36" s="4" t="n">
         <v>0</v>
@@ -4772,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="AH36" s="4" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="AI36" s="4" t="n">
         <v>0</v>
@@ -4787,10 +4787,10 @@
         <v>0</v>
       </c>
       <c r="AM36" s="4" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>1900</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="37">
@@ -5353,7 +5353,7 @@
         <v>1227.9</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>695.88</v>
+        <v>1295.88</v>
       </c>
       <c r="V41" s="4" t="n">
         <v>994.4400000000001</v>
@@ -5371,7 +5371,7 @@
         <v>-1760.43</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>-472.09</v>
+        <v>-1072.09</v>
       </c>
       <c r="AB41" s="4" t="n">
         <v>-173.29</v>
@@ -5383,7 +5383,7 @@
         <v>-236.78</v>
       </c>
       <c r="AE41" s="4" t="n">
-        <v>-2003.28</v>
+        <v>-503.28</v>
       </c>
       <c r="AF41" s="4" t="n">
         <v>406.72</v>
@@ -5392,7 +5392,7 @@
         <v>1126.06</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>842.86</v>
+        <v>-657.14</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>1280.01</v>
@@ -5407,10 +5407,10 @@
         <v>-4720.08</v>
       </c>
       <c r="AM41" s="4" t="n">
-        <v>9078.940000000001</v>
+        <v>9678.940000000001</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>447.15</v>
+        <v>-152.85</v>
       </c>
     </row>
     <row r="42">
@@ -5601,7 +5601,7 @@
         <v>1186.23</v>
       </c>
       <c r="U43" s="4" t="n">
-        <v>654.21</v>
+        <v>1254.21</v>
       </c>
       <c r="V43" s="4" t="n">
         <v>952.77</v>
@@ -5619,7 +5619,7 @@
         <v>-1802.1</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>-547.09</v>
+        <v>-1147.09</v>
       </c>
       <c r="AB43" s="4" t="n">
         <v>-248.29</v>
@@ -5631,7 +5631,7 @@
         <v>-311.78</v>
       </c>
       <c r="AE43" s="4" t="n">
-        <v>-2078.28</v>
+        <v>-578.28</v>
       </c>
       <c r="AF43" s="4" t="n">
         <v>331.72</v>
@@ -5640,7 +5640,7 @@
         <v>1051.06</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>767.86</v>
+        <v>-732.14</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>1205.01</v>
@@ -5655,10 +5655,10 @@
         <v>-4803.42</v>
       </c>
       <c r="AM43" s="4" t="n">
-        <v>8653.940000000001</v>
+        <v>9253.940000000001</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-419.52</v>
+        <v>-1019.52</v>
       </c>
     </row>
     <row r="44">
@@ -6185,7 +6185,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>543</v>
+        <v>657</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -6200,7 +6200,7 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>543</v>
+        <v>657</v>
       </c>
     </row>
     <row r="49">
@@ -6391,7 +6391,7 @@
         <v>778.54</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>1310.56</v>
+        <v>710.5599999999999</v>
       </c>
       <c r="V50" s="4" t="n">
         <v>1061.99</v>
@@ -6409,7 +6409,7 @@
         <v>5598.39</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>5549.96</v>
+        <v>6149.96</v>
       </c>
       <c r="AB50" s="4" t="n">
         <v>4126.11</v>
@@ -6421,7 +6421,7 @@
         <v>4269.53</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>6001.01</v>
+        <v>4501.01</v>
       </c>
       <c r="AF50" s="4" t="n">
         <v>4650.97</v>
@@ -6430,10 +6430,10 @@
         <v>3936.63</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>4264.82</v>
+        <v>5764.82</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>4365.69</v>
+        <v>4479.69</v>
       </c>
       <c r="AJ50" s="4" t="n">
         <v>3825.54</v>
@@ -6445,10 +6445,10 @@
         <v>5889.57</v>
       </c>
       <c r="AM50" s="4" t="n">
-        <v>13931.97</v>
+        <v>13331.97</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>55603.87</v>
+        <v>56317.87</v>
       </c>
     </row>
     <row r="51">
@@ -6515,7 +6515,7 @@
         <v>-438.77</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>-970.79</v>
+        <v>-370.79</v>
       </c>
       <c r="V51" s="4" t="n">
         <v>-672.23</v>
@@ -6533,7 +6533,7 @@
         <v>14906.23</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>14994.58</v>
+        <v>14394.58</v>
       </c>
       <c r="AB51" s="4" t="n">
         <v>-3506.63</v>
@@ -6545,7 +6545,7 @@
         <v>-3570.12</v>
       </c>
       <c r="AE51" s="4" t="n">
-        <v>-5336.62</v>
+        <v>-3836.62</v>
       </c>
       <c r="AF51" s="4" t="n">
         <v>8073.39</v>
@@ -6554,10 +6554,10 @@
         <v>-3207.28</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-3490.47</v>
+        <v>-4990.47</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>-3596.33</v>
+        <v>-3710.33</v>
       </c>
       <c r="AJ51" s="4" t="n">
         <v>-3011.18</v>
@@ -6569,10 +6569,10 @@
         <v>5679.92</v>
       </c>
       <c r="AM51" s="4" t="n">
-        <v>9845.6</v>
+        <v>10445.6</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>4704.13</v>
+        <v>3990.13</v>
       </c>
     </row>
     <row r="52">
@@ -6639,22 +6639,22 @@
         <v>21834.79</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>20864</v>
+        <v>21464</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>20191.77</v>
+        <v>20791.77</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>19937.58</v>
+        <v>20537.58</v>
       </c>
       <c r="X52" s="4" t="n">
-        <v>19677.94</v>
+        <v>20277.94</v>
       </c>
       <c r="Y52" s="4" t="n">
-        <v>18525.53</v>
+        <v>19125.53</v>
       </c>
       <c r="Z52" s="4" t="n">
-        <v>33431.77</v>
+        <v>34031.77</v>
       </c>
       <c r="AA52" s="4" t="n">
         <v>48426.35</v>
@@ -6669,34 +6669,34 @@
         <v>37448.84</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>32112.22</v>
+        <v>33612.22</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>40185.61</v>
+        <v>41685.61</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>36978.33</v>
+        <v>38478.33</v>
       </c>
       <c r="AH52" s="4" t="n">
         <v>33487.85</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>29891.53</v>
+        <v>29777.53</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>26880.35</v>
+        <v>26766.35</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>23229.68</v>
+        <v>23115.68</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
       </c>
       <c r="AM52" s="4" t="n">
-        <v>18525.53</v>
+        <v>19125.53</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>23229.68</v>
+        <v>23115.68</v>
       </c>
     </row>
     <row r="53">
@@ -7122,10 +7122,10 @@
         <v>8679.92</v>
       </c>
       <c r="C7" t="n">
-        <v>18525.53</v>
+        <v>19125.53</v>
       </c>
       <c r="D7" t="n">
-        <v>23229.68</v>
+        <v>23115.68</v>
       </c>
     </row>
     <row r="8">
@@ -7138,10 +7138,10 @@
         <v>9196.59</v>
       </c>
       <c r="C8" t="n">
-        <v>39517.2</v>
+        <v>40117.2</v>
       </c>
       <c r="D8" t="n">
-        <v>44554.68</v>
+        <v>44440.68</v>
       </c>
     </row>
     <row r="9">
@@ -7170,7 +7170,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>543</v>
+        <v>657</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -7186,7 +7186,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>22209.67</v>
+        <v>22323.67</v>
       </c>
       <c r="D11" t="n">
         <v>27666.67</v>
@@ -7202,10 +7202,10 @@
         <v>9196.59</v>
       </c>
       <c r="C12" t="n">
-        <v>17307.53</v>
+        <v>17793.53</v>
       </c>
       <c r="D12" t="n">
-        <v>16888.01</v>
+        <v>16774.01</v>
       </c>
     </row>
     <row r="13">
@@ -7234,10 +7234,10 @@
         <v>-4803.41</v>
       </c>
       <c r="C14" t="n">
-        <v>3307.53</v>
+        <v>3793.53</v>
       </c>
       <c r="D14" t="n">
-        <v>2888.01</v>
+        <v>2774.01</v>
       </c>
     </row>
     <row r="15">
@@ -7250,10 +7250,10 @@
         <v>9196.59</v>
       </c>
       <c r="C15" t="n">
-        <v>17307.53</v>
+        <v>17793.53</v>
       </c>
       <c r="D15" t="n">
-        <v>16888.01</v>
+        <v>16774.01</v>
       </c>
     </row>
   </sheetData>
@@ -11365,7 +11365,7 @@
         <v>0</v>
       </c>
       <c r="U36" s="4" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="V36" s="4" t="n">
         <v>0</v>
@@ -11383,7 +11383,7 @@
         <v>0</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="AB36" s="4" t="n">
         <v>0</v>
@@ -11395,7 +11395,7 @@
         <v>0</v>
       </c>
       <c r="AE36" s="4" t="n">
-        <v>1900</v>
+        <v>400</v>
       </c>
       <c r="AF36" s="4" t="n">
         <v>0</v>
@@ -11404,7 +11404,7 @@
         <v>0</v>
       </c>
       <c r="AH36" s="4" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="AI36" s="4" t="n">
         <v>0</v>
@@ -11419,10 +11419,10 @@
         <v>0</v>
       </c>
       <c r="AM36" s="4" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>1900</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="37">
@@ -11985,7 +11985,7 @@
         <v>2817.73</v>
       </c>
       <c r="U41" s="4" t="n">
-        <v>2323.81</v>
+        <v>2923.81</v>
       </c>
       <c r="V41" s="4" t="n">
         <v>2638.82</v>
@@ -12003,7 +12003,7 @@
         <v>-5457.31</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>-7382.83</v>
+        <v>-7982.83</v>
       </c>
       <c r="AB41" s="4" t="n">
         <v>-5822.34</v>
@@ -12015,7 +12015,7 @@
         <v>-3519.38</v>
       </c>
       <c r="AE41" s="4" t="n">
-        <v>-5106.39</v>
+        <v>-3606.39</v>
       </c>
       <c r="AF41" s="4" t="n">
         <v>-1551.06</v>
@@ -12024,7 +12024,7 @@
         <v>-118.45</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>-346.6</v>
+        <v>-1846.6</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>147.35</v>
@@ -12039,10 +12039,10 @@
         <v>-4720.08</v>
       </c>
       <c r="AM41" s="4" t="n">
-        <v>20599.24</v>
+        <v>21199.24</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-33999.76</v>
+        <v>-34599.76</v>
       </c>
     </row>
     <row r="42">
@@ -12233,7 +12233,7 @@
         <v>2776.06</v>
       </c>
       <c r="U43" s="4" t="n">
-        <v>2282.14</v>
+        <v>2882.14</v>
       </c>
       <c r="V43" s="4" t="n">
         <v>2597.16</v>
@@ -12251,7 +12251,7 @@
         <v>-5579.53</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>-7528.66</v>
+        <v>-8128.66</v>
       </c>
       <c r="AB43" s="4" t="n">
         <v>-5968.17</v>
@@ -12263,7 +12263,7 @@
         <v>-3665.21</v>
       </c>
       <c r="AE43" s="4" t="n">
-        <v>-5252.22</v>
+        <v>-3752.22</v>
       </c>
       <c r="AF43" s="4" t="n">
         <v>-1696.89</v>
@@ -12272,7 +12272,7 @@
         <v>-264.28</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>-492.43</v>
+        <v>-1992.43</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>1.51</v>
@@ -12287,10 +12287,10 @@
         <v>-4803.42</v>
       </c>
       <c r="AM43" s="4" t="n">
-        <v>20174.25</v>
+        <v>20774.25</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-35726.12</v>
+        <v>-36326.12</v>
       </c>
     </row>
     <row r="44">
@@ -12817,7 +12817,7 @@
         <v>0</v>
       </c>
       <c r="AI48" s="4" t="n">
-        <v>2732</v>
+        <v>2846</v>
       </c>
       <c r="AJ48" s="4" t="n">
         <v>0</v>
@@ -12832,7 +12832,7 @@
         <v>0</v>
       </c>
       <c r="AN48" s="4" t="n">
-        <v>2732</v>
+        <v>2846</v>
       </c>
     </row>
     <row r="49">
@@ -13023,7 +13023,7 @@
         <v>990.28</v>
       </c>
       <c r="U50" s="4" t="n">
-        <v>1489.2</v>
+        <v>889.2</v>
       </c>
       <c r="V50" s="4" t="n">
         <v>1224.17</v>
@@ -13041,7 +13041,7 @@
         <v>16016.8</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>17350.49</v>
+        <v>17950.49</v>
       </c>
       <c r="AB50" s="4" t="n">
         <v>15034.9</v>
@@ -13053,7 +13053,7 @@
         <v>15386.81</v>
       </c>
       <c r="AE50" s="4" t="n">
-        <v>16953.77</v>
+        <v>15453.77</v>
       </c>
       <c r="AF50" s="4" t="n">
         <v>16135.06</v>
@@ -13062,10 +13062,10 @@
         <v>14707.44</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>14980.59</v>
+        <v>16480.59</v>
       </c>
       <c r="AI50" s="4" t="n">
-        <v>17213.65</v>
+        <v>17327.65</v>
       </c>
       <c r="AJ50" s="4" t="n">
         <v>14487.24</v>
@@ -13077,10 +13077,10 @@
         <v>5889.57</v>
       </c>
       <c r="AM50" s="4" t="n">
-        <v>17064.08</v>
+        <v>16464.08</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>189782.71</v>
+        <v>190496.71</v>
       </c>
     </row>
     <row r="51">
@@ -13147,7 +13147,7 @@
         <v>-515.6</v>
       </c>
       <c r="U51" s="4" t="n">
-        <v>-1009.53</v>
+        <v>-409.53</v>
       </c>
       <c r="V51" s="4" t="n">
         <v>-694.51</v>
@@ -13165,7 +13165,7 @@
         <v>28642.69</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>19433.84</v>
+        <v>18833.84</v>
       </c>
       <c r="AB51" s="4" t="n">
         <v>-14155.67</v>
@@ -13177,7 +13177,7 @@
         <v>5647.29</v>
       </c>
       <c r="AE51" s="4" t="n">
-        <v>-15939.72</v>
+        <v>-14439.72</v>
       </c>
       <c r="AF51" s="4" t="n">
         <v>16948.94</v>
@@ -13186,10 +13186,10 @@
         <v>-13618.45</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-13846.6</v>
+        <v>-15346.6</v>
       </c>
       <c r="AI51" s="4" t="n">
-        <v>-16084.65</v>
+        <v>-16198.65</v>
       </c>
       <c r="AJ51" s="4" t="n">
         <v>-13318.23</v>
@@ -13201,10 +13201,10 @@
         <v>5679.92</v>
       </c>
       <c r="AM51" s="4" t="n">
-        <v>28032.56</v>
+        <v>28632.56</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>-15648.41</v>
+        <v>-16362.41</v>
       </c>
     </row>
     <row r="52">
@@ -13271,22 +13271,22 @@
         <v>40279.75</v>
       </c>
       <c r="U52" s="4" t="n">
-        <v>39270.22</v>
+        <v>39870.22</v>
       </c>
       <c r="V52" s="4" t="n">
-        <v>38575.71</v>
+        <v>39175.71</v>
       </c>
       <c r="W52" s="4" t="n">
-        <v>38311.57</v>
+        <v>38911.57</v>
       </c>
       <c r="X52" s="4" t="n">
-        <v>38045.76</v>
+        <v>38645.76</v>
       </c>
       <c r="Y52" s="4" t="n">
-        <v>36712.49</v>
+        <v>37312.49</v>
       </c>
       <c r="Z52" s="4" t="n">
-        <v>65355.18</v>
+        <v>65955.17999999999</v>
       </c>
       <c r="AA52" s="4" t="n">
         <v>84789.03</v>
@@ -13301,34 +13301,34 @@
         <v>91478.83</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>75539.11</v>
+        <v>77039.11</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>92488.05</v>
+        <v>93988.05</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>78869.60000000001</v>
+        <v>80369.60000000001</v>
       </c>
       <c r="AH52" s="4" t="n">
         <v>65023</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>48938.35</v>
+        <v>48824.35</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>35620.12</v>
+        <v>35506.12</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>21064.09</v>
+        <v>20950.09</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
       </c>
       <c r="AM52" s="4" t="n">
-        <v>36712.49</v>
+        <v>37312.49</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>21064.09</v>
+        <v>20950.09</v>
       </c>
     </row>
     <row r="53">
@@ -13754,10 +13754,10 @@
         <v>8679.92</v>
       </c>
       <c r="C7" t="n">
-        <v>36712.49</v>
+        <v>37312.49</v>
       </c>
       <c r="D7" t="n">
-        <v>21064.09</v>
+        <v>20950.09</v>
       </c>
     </row>
     <row r="8">
@@ -13770,10 +13770,10 @@
         <v>9196.59</v>
       </c>
       <c r="C8" t="n">
-        <v>81704.16</v>
+        <v>82304.16</v>
       </c>
       <c r="D8" t="n">
-        <v>68079.36</v>
+        <v>67965.36</v>
       </c>
     </row>
     <row r="9">
@@ -13802,7 +13802,7 @@
         <v>0</v>
       </c>
       <c r="C10" t="n">
-        <v>2732</v>
+        <v>2846</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -13818,7 +13818,7 @@
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>55065.33</v>
+        <v>55179.33</v>
       </c>
       <c r="D11" t="n">
         <v>77166.67</v>
@@ -13834,10 +13834,10 @@
         <v>9196.59</v>
       </c>
       <c r="C12" t="n">
-        <v>26638.82</v>
+        <v>27124.82</v>
       </c>
       <c r="D12" t="n">
-        <v>-9087.299999999999</v>
+        <v>-9201.299999999999</v>
       </c>
     </row>
     <row r="13">
@@ -13866,10 +13866,10 @@
         <v>-4803.41</v>
       </c>
       <c r="C14" t="n">
-        <v>12638.82</v>
+        <v>13124.82</v>
       </c>
       <c r="D14" t="n">
-        <v>-23087.3</v>
+        <v>-23201.3</v>
       </c>
     </row>
     <row r="15">
@@ -13882,10 +13882,10 @@
         <v>9196.59</v>
       </c>
       <c r="C15" t="n">
-        <v>26638.82</v>
+        <v>27124.82</v>
       </c>
       <c r="D15" t="n">
-        <v>-9087.299999999999</v>
+        <v>-9201.299999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business plan v6: add CIPA IP Clinic patent consultation details and costs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146q3FtAYmgQ1rtNsNNpdiD
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
@@ -4751,7 +4751,7 @@
         <v>0</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="AB36" s="4" t="n">
         <v>0</v>
@@ -4772,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="AH36" s="4" t="n">
-        <v>1500</v>
+        <v>3350</v>
       </c>
       <c r="AI36" s="4" t="n">
         <v>0</v>
@@ -4790,7 +4790,7 @@
         <v>900</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>2500</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="37">
@@ -5371,7 +5371,7 @@
         <v>-1760.43</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>-1072.09</v>
+        <v>-472.09</v>
       </c>
       <c r="AB41" s="4" t="n">
         <v>-173.29</v>
@@ -5392,7 +5392,7 @@
         <v>1126.06</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>-657.14</v>
+        <v>-2507.14</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>1280.01</v>
@@ -5410,7 +5410,7 @@
         <v>9678.940000000001</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-152.85</v>
+        <v>-1402.85</v>
       </c>
     </row>
     <row r="42">
@@ -5619,7 +5619,7 @@
         <v>-1802.1</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>-1147.09</v>
+        <v>-547.09</v>
       </c>
       <c r="AB43" s="4" t="n">
         <v>-248.29</v>
@@ -5640,7 +5640,7 @@
         <v>1051.06</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>-732.14</v>
+        <v>-2582.14</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>1205.01</v>
@@ -5658,7 +5658,7 @@
         <v>9253.940000000001</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-1019.52</v>
+        <v>-2269.52</v>
       </c>
     </row>
     <row r="44">
@@ -6409,7 +6409,7 @@
         <v>5598.39</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>6149.96</v>
+        <v>5549.96</v>
       </c>
       <c r="AB50" s="4" t="n">
         <v>4126.11</v>
@@ -6430,7 +6430,7 @@
         <v>3936.63</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>5764.82</v>
+        <v>7614.82</v>
       </c>
       <c r="AI50" s="4" t="n">
         <v>4479.69</v>
@@ -6448,7 +6448,7 @@
         <v>13331.97</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>56317.87</v>
+        <v>57567.87</v>
       </c>
     </row>
     <row r="51">
@@ -6533,7 +6533,7 @@
         <v>14906.23</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>14394.58</v>
+        <v>14994.58</v>
       </c>
       <c r="AB51" s="4" t="n">
         <v>-3506.63</v>
@@ -6554,7 +6554,7 @@
         <v>-3207.28</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-4990.47</v>
+        <v>-6840.47</v>
       </c>
       <c r="AI51" s="4" t="n">
         <v>-3710.33</v>
@@ -6572,7 +6572,7 @@
         <v>10445.6</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>3990.13</v>
+        <v>2740.13</v>
       </c>
     </row>
     <row r="52">
@@ -6657,37 +6657,37 @@
         <v>34031.77</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>48426.35</v>
+        <v>49026.35</v>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>44919.72</v>
+        <v>45519.72</v>
       </c>
       <c r="AC52" s="4" t="n">
-        <v>41018.95</v>
+        <v>41618.95</v>
       </c>
       <c r="AD52" s="4" t="n">
-        <v>37448.84</v>
+        <v>38048.84</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>33612.22</v>
+        <v>34212.22</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>41685.61</v>
+        <v>42285.61</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>38478.33</v>
+        <v>39078.33</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>33487.85</v>
+        <v>32237.85</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>29777.53</v>
+        <v>28527.53</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>26766.35</v>
+        <v>25516.35</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>23115.68</v>
+        <v>21865.68</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
@@ -6696,7 +6696,7 @@
         <v>19125.53</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>23115.68</v>
+        <v>21865.68</v>
       </c>
     </row>
     <row r="53">
@@ -7125,7 +7125,7 @@
         <v>19125.53</v>
       </c>
       <c r="D7" t="n">
-        <v>23115.68</v>
+        <v>21865.68</v>
       </c>
     </row>
     <row r="8">
@@ -7141,7 +7141,7 @@
         <v>40117.2</v>
       </c>
       <c r="D8" t="n">
-        <v>44440.68</v>
+        <v>43190.68</v>
       </c>
     </row>
     <row r="9">
@@ -7205,7 +7205,7 @@
         <v>17793.53</v>
       </c>
       <c r="D12" t="n">
-        <v>16774.01</v>
+        <v>15524.01</v>
       </c>
     </row>
     <row r="13">
@@ -7237,7 +7237,7 @@
         <v>3793.53</v>
       </c>
       <c r="D14" t="n">
-        <v>2774.01</v>
+        <v>1524.01</v>
       </c>
     </row>
     <row r="15">
@@ -7253,7 +7253,7 @@
         <v>17793.53</v>
       </c>
       <c r="D15" t="n">
-        <v>16774.01</v>
+        <v>15524.01</v>
       </c>
     </row>
   </sheetData>
@@ -11383,7 +11383,7 @@
         <v>0</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="AB36" s="4" t="n">
         <v>0</v>
@@ -11404,7 +11404,7 @@
         <v>0</v>
       </c>
       <c r="AH36" s="4" t="n">
-        <v>1500</v>
+        <v>3350</v>
       </c>
       <c r="AI36" s="4" t="n">
         <v>0</v>
@@ -11422,7 +11422,7 @@
         <v>900</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>2500</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="37">
@@ -12003,7 +12003,7 @@
         <v>-5457.31</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>-7982.83</v>
+        <v>-7382.83</v>
       </c>
       <c r="AB41" s="4" t="n">
         <v>-5822.34</v>
@@ -12024,7 +12024,7 @@
         <v>-118.45</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>-1846.6</v>
+        <v>-3696.6</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>147.35</v>
@@ -12042,7 +12042,7 @@
         <v>21199.24</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-34599.76</v>
+        <v>-35849.76</v>
       </c>
     </row>
     <row r="42">
@@ -12251,7 +12251,7 @@
         <v>-5579.53</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>-8128.66</v>
+        <v>-7528.66</v>
       </c>
       <c r="AB43" s="4" t="n">
         <v>-5968.17</v>
@@ -12272,7 +12272,7 @@
         <v>-264.28</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>-1992.43</v>
+        <v>-3842.43</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>1.51</v>
@@ -12290,7 +12290,7 @@
         <v>20774.25</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-36326.12</v>
+        <v>-37576.12</v>
       </c>
     </row>
     <row r="44">
@@ -13041,7 +13041,7 @@
         <v>16016.8</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>17950.49</v>
+        <v>17350.49</v>
       </c>
       <c r="AB50" s="4" t="n">
         <v>15034.9</v>
@@ -13062,7 +13062,7 @@
         <v>14707.44</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>16480.59</v>
+        <v>18330.59</v>
       </c>
       <c r="AI50" s="4" t="n">
         <v>17327.65</v>
@@ -13080,7 +13080,7 @@
         <v>16464.08</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>190496.71</v>
+        <v>191746.71</v>
       </c>
     </row>
     <row r="51">
@@ -13165,7 +13165,7 @@
         <v>28642.69</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>18833.84</v>
+        <v>19433.84</v>
       </c>
       <c r="AB51" s="4" t="n">
         <v>-14155.67</v>
@@ -13186,7 +13186,7 @@
         <v>-13618.45</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-15346.6</v>
+        <v>-17196.6</v>
       </c>
       <c r="AI51" s="4" t="n">
         <v>-16198.65</v>
@@ -13204,7 +13204,7 @@
         <v>28632.56</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>-16362.41</v>
+        <v>-17612.41</v>
       </c>
     </row>
     <row r="52">
@@ -13289,37 +13289,37 @@
         <v>65955.17999999999</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>84789.03</v>
+        <v>85389.03</v>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>70633.36</v>
+        <v>71233.36</v>
       </c>
       <c r="AC52" s="4" t="n">
-        <v>85831.53999999999</v>
+        <v>86431.53999999999</v>
       </c>
       <c r="AD52" s="4" t="n">
-        <v>91478.83</v>
+        <v>92078.83</v>
       </c>
       <c r="AE52" s="4" t="n">
-        <v>77039.11</v>
+        <v>77639.11</v>
       </c>
       <c r="AF52" s="4" t="n">
-        <v>93988.05</v>
+        <v>94588.05</v>
       </c>
       <c r="AG52" s="4" t="n">
-        <v>80369.60000000001</v>
+        <v>80969.60000000001</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>65023</v>
+        <v>63773</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>48824.35</v>
+        <v>47574.35</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>35506.12</v>
+        <v>34256.12</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>20950.09</v>
+        <v>19700.09</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
@@ -13328,7 +13328,7 @@
         <v>37312.49</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>20950.09</v>
+        <v>19700.09</v>
       </c>
     </row>
     <row r="53">
@@ -13757,7 +13757,7 @@
         <v>37312.49</v>
       </c>
       <c r="D7" t="n">
-        <v>20950.09</v>
+        <v>19700.09</v>
       </c>
     </row>
     <row r="8">
@@ -13773,7 +13773,7 @@
         <v>82304.16</v>
       </c>
       <c r="D8" t="n">
-        <v>67965.36</v>
+        <v>66715.36</v>
       </c>
     </row>
     <row r="9">
@@ -13837,7 +13837,7 @@
         <v>27124.82</v>
       </c>
       <c r="D12" t="n">
-        <v>-9201.299999999999</v>
+        <v>-10451.3</v>
       </c>
     </row>
     <row r="13">
@@ -13869,7 +13869,7 @@
         <v>13124.82</v>
       </c>
       <c r="D14" t="n">
-        <v>-23201.3</v>
+        <v>-24451.3</v>
       </c>
     </row>
     <row r="15">
@@ -13885,7 +13885,7 @@
         <v>27124.82</v>
       </c>
       <c r="D15" t="n">
-        <v>-9201.299999999999</v>
+        <v>-10451.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Business plan v6: patent exploration after three-year endorsement and university conversion
Patent costs removed from the 36-month forecast; Section 3.4, SWOT, risk
table and P&L commentary updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146q3FtAYmgQ1rtNsNNpdiD
</commit_message>
<xml_diff>
--- a/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
+++ b/visa_appendices/DEQUAD_Financial_Model_v6.xlsx
@@ -4772,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="AH36" s="4" t="n">
-        <v>3350</v>
+        <v>0</v>
       </c>
       <c r="AI36" s="4" t="n">
         <v>0</v>
@@ -4790,7 +4790,7 @@
         <v>900</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>3750</v>
+        <v>400</v>
       </c>
     </row>
     <row r="37">
@@ -5392,7 +5392,7 @@
         <v>1126.06</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>-2507.14</v>
+        <v>842.86</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>1280.01</v>
@@ -5410,7 +5410,7 @@
         <v>9678.940000000001</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-1402.85</v>
+        <v>1947.15</v>
       </c>
     </row>
     <row r="42">
@@ -5640,7 +5640,7 @@
         <v>1051.06</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>-2582.14</v>
+        <v>767.86</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>1205.01</v>
@@ -5658,7 +5658,7 @@
         <v>9253.940000000001</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-2269.52</v>
+        <v>1080.48</v>
       </c>
     </row>
     <row r="44">
@@ -6430,7 +6430,7 @@
         <v>3936.63</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>7614.82</v>
+        <v>4264.82</v>
       </c>
       <c r="AI50" s="4" t="n">
         <v>4479.69</v>
@@ -6448,7 +6448,7 @@
         <v>13331.97</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>57567.87</v>
+        <v>54217.87</v>
       </c>
     </row>
     <row r="51">
@@ -6554,7 +6554,7 @@
         <v>-3207.28</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-6840.47</v>
+        <v>-3490.47</v>
       </c>
       <c r="AI51" s="4" t="n">
         <v>-3710.33</v>
@@ -6572,7 +6572,7 @@
         <v>10445.6</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>2740.13</v>
+        <v>6090.13</v>
       </c>
     </row>
     <row r="52">
@@ -6678,16 +6678,16 @@
         <v>39078.33</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>32237.85</v>
+        <v>35587.85</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>28527.53</v>
+        <v>31877.53</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>25516.35</v>
+        <v>28866.35</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>21865.68</v>
+        <v>25215.68</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
@@ -6696,7 +6696,7 @@
         <v>19125.53</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>21865.68</v>
+        <v>25215.68</v>
       </c>
     </row>
     <row r="53">
@@ -7125,7 +7125,7 @@
         <v>19125.53</v>
       </c>
       <c r="D7" t="n">
-        <v>21865.68</v>
+        <v>25215.68</v>
       </c>
     </row>
     <row r="8">
@@ -7141,7 +7141,7 @@
         <v>40117.2</v>
       </c>
       <c r="D8" t="n">
-        <v>43190.68</v>
+        <v>46540.68</v>
       </c>
     </row>
     <row r="9">
@@ -7173,7 +7173,7 @@
         <v>657</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11">
@@ -7189,7 +7189,7 @@
         <v>22323.67</v>
       </c>
       <c r="D11" t="n">
-        <v>27666.67</v>
+        <v>27808.67</v>
       </c>
     </row>
     <row r="12">
@@ -7205,7 +7205,7 @@
         <v>17793.53</v>
       </c>
       <c r="D12" t="n">
-        <v>15524.01</v>
+        <v>18732.01</v>
       </c>
     </row>
     <row r="13">
@@ -7237,7 +7237,7 @@
         <v>3793.53</v>
       </c>
       <c r="D14" t="n">
-        <v>1524.01</v>
+        <v>4732.01</v>
       </c>
     </row>
     <row r="15">
@@ -7253,7 +7253,7 @@
         <v>17793.53</v>
       </c>
       <c r="D15" t="n">
-        <v>15524.01</v>
+        <v>18732.01</v>
       </c>
     </row>
   </sheetData>
@@ -11404,7 +11404,7 @@
         <v>0</v>
       </c>
       <c r="AH36" s="4" t="n">
-        <v>3350</v>
+        <v>0</v>
       </c>
       <c r="AI36" s="4" t="n">
         <v>0</v>
@@ -11422,7 +11422,7 @@
         <v>900</v>
       </c>
       <c r="AN36" s="4" t="n">
-        <v>3750</v>
+        <v>400</v>
       </c>
     </row>
     <row r="37">
@@ -12024,7 +12024,7 @@
         <v>-118.45</v>
       </c>
       <c r="AH41" s="4" t="n">
-        <v>-3696.6</v>
+        <v>-346.6</v>
       </c>
       <c r="AI41" s="4" t="n">
         <v>147.35</v>
@@ -12042,7 +12042,7 @@
         <v>21199.24</v>
       </c>
       <c r="AN41" s="4" t="n">
-        <v>-35849.76</v>
+        <v>-32499.76</v>
       </c>
     </row>
     <row r="42">
@@ -12272,7 +12272,7 @@
         <v>-264.28</v>
       </c>
       <c r="AH43" s="4" t="n">
-        <v>-3842.43</v>
+        <v>-492.43</v>
       </c>
       <c r="AI43" s="4" t="n">
         <v>1.51</v>
@@ -12290,7 +12290,7 @@
         <v>20774.25</v>
       </c>
       <c r="AN43" s="4" t="n">
-        <v>-37576.12</v>
+        <v>-34226.12</v>
       </c>
     </row>
     <row r="44">
@@ -13062,7 +13062,7 @@
         <v>14707.44</v>
       </c>
       <c r="AH50" s="4" t="n">
-        <v>18330.59</v>
+        <v>14980.59</v>
       </c>
       <c r="AI50" s="4" t="n">
         <v>17327.65</v>
@@ -13080,7 +13080,7 @@
         <v>16464.08</v>
       </c>
       <c r="AN50" s="4" t="n">
-        <v>191746.71</v>
+        <v>188396.71</v>
       </c>
     </row>
     <row r="51">
@@ -13186,7 +13186,7 @@
         <v>-13618.45</v>
       </c>
       <c r="AH51" s="4" t="n">
-        <v>-17196.6</v>
+        <v>-13846.6</v>
       </c>
       <c r="AI51" s="4" t="n">
         <v>-16198.65</v>
@@ -13204,7 +13204,7 @@
         <v>28632.56</v>
       </c>
       <c r="AN51" s="4" t="n">
-        <v>-17612.41</v>
+        <v>-14262.41</v>
       </c>
     </row>
     <row r="52">
@@ -13310,16 +13310,16 @@
         <v>80969.60000000001</v>
       </c>
       <c r="AH52" s="4" t="n">
-        <v>63773</v>
+        <v>67123</v>
       </c>
       <c r="AI52" s="4" t="n">
-        <v>47574.35</v>
+        <v>50924.35</v>
       </c>
       <c r="AJ52" s="4" t="n">
-        <v>34256.12</v>
+        <v>37606.12</v>
       </c>
       <c r="AK52" s="4" t="n">
-        <v>19700.09</v>
+        <v>23050.09</v>
       </c>
       <c r="AL52" s="4" t="n">
         <v>8679.92</v>
@@ -13328,7 +13328,7 @@
         <v>37312.49</v>
       </c>
       <c r="AN52" s="4" t="n">
-        <v>19700.09</v>
+        <v>23050.09</v>
       </c>
     </row>
     <row r="53">
@@ -13757,7 +13757,7 @@
         <v>37312.49</v>
       </c>
       <c r="D7" t="n">
-        <v>19700.09</v>
+        <v>23050.09</v>
       </c>
     </row>
     <row r="8">
@@ -13773,7 +13773,7 @@
         <v>82304.16</v>
       </c>
       <c r="D8" t="n">
-        <v>66715.36</v>
+        <v>70065.36</v>
       </c>
     </row>
     <row r="9">
@@ -13837,7 +13837,7 @@
         <v>27124.82</v>
       </c>
       <c r="D12" t="n">
-        <v>-10451.3</v>
+        <v>-7101.3</v>
       </c>
     </row>
     <row r="13">
@@ -13869,7 +13869,7 @@
         <v>13124.82</v>
       </c>
       <c r="D14" t="n">
-        <v>-24451.3</v>
+        <v>-21101.3</v>
       </c>
     </row>
     <row r="15">
@@ -13885,7 +13885,7 @@
         <v>27124.82</v>
       </c>
       <c r="D15" t="n">
-        <v>-10451.3</v>
+        <v>-7101.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>